<commit_message>
Audit fixes: shared Baskin/Cinnabon locations + portal regenerator rewrite
- build_database.py: BS04/16/31/37 marcados BASKIN ROBBINS / CINNABON,
  nombre tomado de entrada CN del PRESUPUESTO; auditoría reconoce CN compartidas
- index.html: regenerarBaseDatos() reescrito para replicar exactamente la lógica
  Python (3 fuentes, 198 locales, recarga incluye mantt). Detección dinámica de
  columnas (SheetJS recorta columna A vacía del PRESUPUESTO). Verificado E2E:
  898 extintores, 198 locales, $19,323.30 — idéntico al script Python
- Texto del portal actualizado (198 locales, fórmula no aditiva)

https://claude.ai/code/session_0181v9mDMYaZBVAjFuZBPUmm
</commit_message>
<xml_diff>
--- a/BASE_DATOS_KFC.xlsx
+++ b/BASE_DATOS_KFC.xlsx
@@ -460,7 +460,7 @@
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
     <col width="47" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
@@ -8503,7 +8503,7 @@
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>BASKIN ROBBINS</t>
+          <t>BASKIN ROBBINS / CINNABON</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
@@ -8566,7 +8566,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>BASKIN ROBBINS</t>
+          <t>BASKIN ROBBINS / CINNABON</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -8692,10 +8692,14 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>BASKIN ROBBINS</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr"/>
+          <t>BASKIN ROBBINS / CINNABON</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>CN31 - RIOCENTRO CEIBOS</t>
+        </is>
+      </c>
       <c r="E131" t="inlineStr">
         <is>
           <t>FEBRERO</t>
@@ -12846,7 +12850,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>BASKIN ROBBINS</t>
+          <t>BASKIN ROBBINS / CINNABON</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -19173,7 +19177,7 @@
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>BASKIN ROBBINS</t>
+          <t>BASKIN ROBBINS / CINNABON</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
@@ -56670,7 +56674,7 @@
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
     <col width="47" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -57957,7 +57961,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>BASKIN ROBBINS</t>
+          <t>BASKIN ROBBINS / CINNABON</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -58057,10 +58061,14 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>BASKIN ROBBINS</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr"/>
+          <t>BASKIN ROBBINS / CINNABON</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>CN31 - RIOCENTRO CEIBOS</t>
+        </is>
+      </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
           <t>FEBRERO</t>
@@ -58903,7 +58911,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>BASKIN ROBBINS</t>
+          <t>BASKIN ROBBINS / CINNABON</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -60103,7 +60111,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>BASKIN ROBBINS</t>
+          <t>BASKIN ROBBINS / CINNABON</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -66639,10 +66647,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
   </cols>
@@ -66667,168 +66675,100 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EN_PRESUP_SIN_EXTINTOR</t>
+          <t>EN_MATRIZ_SIN_PRESUP</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CN004</t>
+          <t>BS031</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CN04EC – CINNABON – CN04 - MALL DEL SOL</t>
+          <t>Nuevo local no en PRESUPUESTO 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EN_PRESUP_SIN_EXTINTOR</t>
+          <t>EN_MATRIZ_SIN_PRESUP</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CN016</t>
+          <t>K192</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CN16EC – CINNABON – CN16 - PUNTILLA</t>
+          <t>Nuevo local no en PRESUPUESTO 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EN_PRESUP_SIN_EXTINTOR</t>
+          <t>EN_MATRIZ_SIN_PRESUP</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CN031</t>
+          <t>K194</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CN31EC – CINNABON – CN31 - RIOCENTRO CEIBOS</t>
+          <t>Nuevo local no en PRESUPUESTO 2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EN_PRESUP_SIN_EXTINTOR</t>
+          <t>EN_MATRIZ_SIN_PRESUP</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CN037</t>
+          <t>V091</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CN37EC – CINNABON – CN37 - EL DORADO</t>
+          <t>Nuevo local no en PRESUPUESTO 2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>EN_MATRIZ_SIN_PRESUP</t>
+          <t>FUSIONADO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BS031</t>
+          <t>H068</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Nuevo local no en PRESUPUESTO 2026</t>
+          <t>Heladerías Mall del Norte fusionado en K172 (extintor 'heladería' incluido en K172)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EN_MATRIZ_SIN_PRESUP</t>
+          <t>ELIMINADO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>K192</t>
+          <t>G042</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
-        <is>
-          <t>Nuevo local no en PRESUPUESTO 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>EN_MATRIZ_SIN_PRESUP</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>K194</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Nuevo local no en PRESUPUESTO 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>EN_MATRIZ_SIN_PRESUP</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>V091</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Nuevo local no en PRESUPUESTO 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>FUSIONADO</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>H068</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Heladerías Mall del Norte fusionado en K172 (extintor 'heladería' incluido en K172)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>ELIMINADO</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>G042</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
         <is>
           <t>GUS Quito Aguirre – local cerrado, excluido de la base</t>
         </is>

</xml_diff>

<commit_message>
Corrige viáticos K79 $40→$39, B1 servicio mixto OCT, omite ventas y COTIZACION1464 del reporte
- build_database.py: K79 viáticos $40 → $39
- build_database.py: MIXED_SERVICE_MANTT para B1 Sports Bar OCT
  (50CO2 → MANTT $20, resto → RECARGA; COBRO_ANUAL=$77.20 antes $102.20)
- revision_cotizaciones.py: VENTAS omitidas completamente del reporte (no se muestra fila)
- revision_cotizaciones.py: SKIP_FILES {COTIZACION1464} — R10 servicio aparte, ignorado
- revision_cotizaciones.py: comparar COBRO_ANUAL (no TOTAL_RECARGA) en meses de recarga
  (B1 pasa de diff=22.9% a diff=2.1% al usar el cobro mixto correcto)
- Resultado: 197 locales, $20,108.20 cobro anual, 101 OK / 14 INCONSISTENCIAS / 5 COT_DEBE_RECARGA

https://claude.ai/code/session_017rdRDT2VUBvb4GkrdojQaa
</commit_message>
<xml_diff>
--- a/BASE_DATOS_KFC.xlsx
+++ b/BASE_DATOS_KFC.xlsx
@@ -21045,10 +21045,10 @@
       </c>
       <c r="F597" s="8" t="inlineStr"/>
       <c r="G597" s="9" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H597" s="9" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I597" s="8" t="n"/>
       <c r="J597" s="8" t="n"/>
@@ -21065,14 +21065,14 @@
       <c r="E598" s="4" t="inlineStr"/>
       <c r="F598" s="4" t="inlineStr">
         <is>
-          <t>5 ext. + movil.$40.00</t>
+          <t>5 ext. + movil.$39.00</t>
         </is>
       </c>
       <c r="G598" s="7" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H598" s="7" t="n">
-        <v>122.6</v>
+        <v>121.6</v>
       </c>
       <c r="I598" s="4" t="inlineStr"/>
       <c r="J598" s="4" t="inlineStr"/>
@@ -49396,13 +49396,13 @@
         <v>5</v>
       </c>
       <c r="F90" s="12" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G90" s="12" t="n">
-        <v>122.6</v>
+        <v>121.6</v>
       </c>
       <c r="H90" s="12" t="n">
-        <v>122.6</v>
+        <v>121.6</v>
       </c>
       <c r="I90" s="11" t="n">
         <v>2024</v>
@@ -51802,7 +51802,7 @@
         <v>102.2</v>
       </c>
       <c r="H150" s="12" t="n">
-        <v>102.2</v>
+        <v>77.2</v>
       </c>
       <c r="I150" s="11" t="n">
         <v>2023</v>
@@ -53736,13 +53736,13 @@
         <v>906</v>
       </c>
       <c r="F199" s="15" t="n">
-        <v>7073.3</v>
+        <v>7072.3</v>
       </c>
       <c r="G199" s="15" t="n">
-        <v>20134.2</v>
+        <v>20133.2</v>
       </c>
       <c r="H199" s="15" t="n">
-        <v>20134.2</v>
+        <v>20108.2</v>
       </c>
       <c r="I199" s="1" t="inlineStr"/>
       <c r="J199" s="1" t="inlineStr"/>

</xml_diff>

<commit_message>
Add 13 SUSHICORP locales (KN01–KN13) to BASE_DATOS_KFC.xlsx
Adds Kobe and Noe restaurant chain to the database:
- 10 Kobe locales + 3 Noe locales across GYE
- Individual extintor records sourced from MATRIZ SUSHICORP (Dropbox)
- Service months from PROYECCION INGRESOS MENSUAL 2026 (Dropbox)
- Total: 210 locales, 968 extintores database-wide

https://claude.ai/code/session_017rdRDT2VUBvb4GkrdojQaa
</commit_message>
<xml_diff>
--- a/BASE_DATOS_KFC.xlsx
+++ b/BASE_DATOS_KFC.xlsx
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1317"/>
+  <dimension ref="A1:K1405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -45573,7 +45573,2246 @@
       <c r="I1317" s="4" t="inlineStr"/>
       <c r="J1317" s="4" t="inlineStr"/>
     </row>
-    <row r="1318" ht="8" customHeight="1"/>
+    <row r="1318" ht="8" customHeight="1">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>KN01 - NOE MALL DEL SOL</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>FEBRERO</t>
+        </is>
+      </c>
+      <c r="D1318" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1318" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1318" t="inlineStr">
+        <is>
+          <t>50 LBS</t>
+        </is>
+      </c>
+      <c r="G1318" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1318" t="n">
+        <v>20</v>
+      </c>
+      <c r="I1318" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1318" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="D1319" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1319" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1319" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1319" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1319" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1319" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1319" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="D1320" t="inlineStr">
+        <is>
+          <t>OFICINA</t>
+        </is>
+      </c>
+      <c r="E1320" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1320" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1320" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1320" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1320" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1320" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="D1321" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1321" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1321" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1321" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1321" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1321" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1321" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="D1322" t="inlineStr">
+        <is>
+          <t>GABINETE ENTRADA</t>
+        </is>
+      </c>
+      <c r="E1322" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1322" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1322" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1322" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1322" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1322" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="D1323" t="inlineStr">
+        <is>
+          <t>BODEGA</t>
+        </is>
+      </c>
+      <c r="E1323" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1323" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1323" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1323" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1323" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1323" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>TOTALES  SUSHICORP – KN01 - NOE MALL DEL SOL</t>
+        </is>
+      </c>
+      <c r="F1324" t="inlineStr">
+        <is>
+          <t>6 ext.</t>
+        </is>
+      </c>
+      <c r="G1324" t="n">
+        <v>40</v>
+      </c>
+      <c r="H1324" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1325"/>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>KN02 - NOE BOCCA SAMBO</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>FEBRERO</t>
+        </is>
+      </c>
+      <c r="D1326" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1326" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1326" t="inlineStr">
+        <is>
+          <t>50 LBS</t>
+        </is>
+      </c>
+      <c r="G1326" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1326" t="n">
+        <v>20</v>
+      </c>
+      <c r="I1326" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1326" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="D1327" t="inlineStr">
+        <is>
+          <t>SALON</t>
+        </is>
+      </c>
+      <c r="E1327" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1327" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1327" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1327" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1327" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1327" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="D1328" t="inlineStr">
+        <is>
+          <t>BODEGA</t>
+        </is>
+      </c>
+      <c r="E1328" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1328" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1328" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1328" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1328" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1328" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="D1329" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1329" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1329" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1329" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1329" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1329" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1329" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr">
+        <is>
+          <t>TOTALES  SUSHICORP – KN02 - NOE BOCCA SAMBO</t>
+        </is>
+      </c>
+      <c r="F1330" t="inlineStr">
+        <is>
+          <t>4 ext.</t>
+        </is>
+      </c>
+      <c r="G1330" t="n">
+        <v>32</v>
+      </c>
+      <c r="H1330" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1331"/>
+    <row r="1332">
+      <c r="A1332" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>KN03 - KOBE PLANTA</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>FEBRERO</t>
+        </is>
+      </c>
+      <c r="D1332" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
+      <c r="E1332" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1332" t="inlineStr">
+        <is>
+          <t>50 LBS</t>
+        </is>
+      </c>
+      <c r="G1332" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1332" t="n">
+        <v>20</v>
+      </c>
+      <c r="I1332" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1332" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="D1333" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
+      <c r="E1333" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1333" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1333" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1333" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1333" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1333" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="D1334" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
+      <c r="E1334" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1334" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1334" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1334" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1334" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1334" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="D1335" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
+      <c r="E1335" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1335" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1335" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1335" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1335" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1335" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="D1336" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
+      <c r="E1336" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1336" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1336" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1336" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1336" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1336" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="D1337" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
+      <c r="E1337" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1337" t="inlineStr">
+        <is>
+          <t>5 LBS</t>
+        </is>
+      </c>
+      <c r="G1337" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1337" t="n">
+        <v>2</v>
+      </c>
+      <c r="I1337" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1337" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="D1338" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
+      <c r="E1338" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1338" t="inlineStr">
+        <is>
+          <t>5 LBS</t>
+        </is>
+      </c>
+      <c r="G1338" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1338" t="n">
+        <v>2</v>
+      </c>
+      <c r="I1338" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1338" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="D1339" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
+      <c r="E1339" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1339" t="inlineStr">
+        <is>
+          <t>5 LBS</t>
+        </is>
+      </c>
+      <c r="G1339" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1339" t="n">
+        <v>2</v>
+      </c>
+      <c r="I1339" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1339" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="D1340" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
+      <c r="E1340" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1340" t="inlineStr">
+        <is>
+          <t>5 LBS</t>
+        </is>
+      </c>
+      <c r="G1340" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1340" t="n">
+        <v>2</v>
+      </c>
+      <c r="I1340" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1340" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="D1341" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
+      <c r="E1341" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1341" t="inlineStr">
+        <is>
+          <t>5 LBS</t>
+        </is>
+      </c>
+      <c r="G1341" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1341" t="n">
+        <v>2</v>
+      </c>
+      <c r="I1341" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1341" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="D1342" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
+      <c r="E1342" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1342" t="inlineStr">
+        <is>
+          <t>20 LBS</t>
+        </is>
+      </c>
+      <c r="G1342" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1342" t="n">
+        <v>8</v>
+      </c>
+      <c r="I1342" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1342" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="D1343" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
+      <c r="E1343" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1343" t="inlineStr">
+        <is>
+          <t>20 LBS</t>
+        </is>
+      </c>
+      <c r="G1343" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1343" t="n">
+        <v>8</v>
+      </c>
+      <c r="I1343" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1343" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="D1344" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
+      <c r="E1344" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1344" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1344" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1344" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1344" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1344" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="D1345" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
+      <c r="E1345" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1345" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1345" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1345" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1345" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1345" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="D1346" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
+      <c r="E1346" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1346" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1346" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1346" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1346" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1346" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="D1347" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
+      <c r="E1347" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1347" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1347" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1347" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1347" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1347" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="inlineStr">
+        <is>
+          <t>TOTALES  SUSHICORP – KN03 - KOBE PLANTA</t>
+        </is>
+      </c>
+      <c r="F1348" t="inlineStr">
+        <is>
+          <t>16 ext.</t>
+        </is>
+      </c>
+      <c r="G1348" t="n">
+        <v>78</v>
+      </c>
+      <c r="H1348" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="1349"/>
+    <row r="1350">
+      <c r="A1350" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="B1350" t="inlineStr">
+        <is>
+          <t>KN04 - KOBE SUPERCINES ORELLANA</t>
+        </is>
+      </c>
+      <c r="C1350" t="inlineStr">
+        <is>
+          <t>MARZO</t>
+        </is>
+      </c>
+      <c r="D1350" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1350" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1350" t="inlineStr">
+        <is>
+          <t>50 LBS</t>
+        </is>
+      </c>
+      <c r="G1350" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1350" t="n">
+        <v>20</v>
+      </c>
+      <c r="I1350" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1350" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="D1351" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1351" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1351" t="inlineStr">
+        <is>
+          <t>5 LBS</t>
+        </is>
+      </c>
+      <c r="G1351" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1351" t="n">
+        <v>2</v>
+      </c>
+      <c r="I1351" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1351" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="D1352" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1352" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1352" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1352" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1352" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1352" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1352" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="inlineStr">
+        <is>
+          <t>TOTALES  SUSHICORP – KN04 - KOBE SUPERCINES ORELLANA</t>
+        </is>
+      </c>
+      <c r="F1353" t="inlineStr">
+        <is>
+          <t>3 ext.</t>
+        </is>
+      </c>
+      <c r="G1353" t="n">
+        <v>26</v>
+      </c>
+      <c r="H1353" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1354"/>
+    <row r="1355">
+      <c r="A1355" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="B1355" t="inlineStr">
+        <is>
+          <t>KN05 - KOBE MALL DEL SOL</t>
+        </is>
+      </c>
+      <c r="C1355" t="inlineStr">
+        <is>
+          <t>AGOSTO</t>
+        </is>
+      </c>
+      <c r="D1355" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1355" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1355" t="inlineStr">
+        <is>
+          <t>50 LBS</t>
+        </is>
+      </c>
+      <c r="G1355" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1355" t="n">
+        <v>20</v>
+      </c>
+      <c r="I1355" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1355" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="D1356" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1356" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1356" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1356" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1356" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1356" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1356" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" t="inlineStr">
+        <is>
+          <t>TOTALES  SUSHICORP – KN05 - KOBE MALL DEL SOL</t>
+        </is>
+      </c>
+      <c r="F1357" t="inlineStr">
+        <is>
+          <t>2 ext.</t>
+        </is>
+      </c>
+      <c r="G1357" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1357" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="1358"/>
+    <row r="1359">
+      <c r="A1359" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="B1359" t="inlineStr">
+        <is>
+          <t>KN06 - KOBE PLAZA BATAN</t>
+        </is>
+      </c>
+      <c r="C1359" t="inlineStr">
+        <is>
+          <t>AGOSTO</t>
+        </is>
+      </c>
+      <c r="D1359" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1359" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1359" t="inlineStr">
+        <is>
+          <t>50 LBS</t>
+        </is>
+      </c>
+      <c r="G1359" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1359" t="n">
+        <v>20</v>
+      </c>
+      <c r="I1359" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1359" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="D1360" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1360" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1360" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1360" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1360" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1360" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1360" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="D1361" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1361" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1361" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1361" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1361" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1361" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1361" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" t="inlineStr">
+        <is>
+          <t>TOTALES  SUSHICORP – KN06 - KOBE PLAZA BATAN</t>
+        </is>
+      </c>
+      <c r="F1362" t="inlineStr">
+        <is>
+          <t>3 ext.</t>
+        </is>
+      </c>
+      <c r="G1362" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1362" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="1363"/>
+    <row r="1364">
+      <c r="A1364" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="B1364" t="inlineStr">
+        <is>
+          <t>KN07 - KOBE MALL DEL NORTE</t>
+        </is>
+      </c>
+      <c r="C1364" t="inlineStr">
+        <is>
+          <t>AGOSTO</t>
+        </is>
+      </c>
+      <c r="D1364" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1364" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1364" t="inlineStr">
+        <is>
+          <t>50 LBS</t>
+        </is>
+      </c>
+      <c r="G1364" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1364" t="n">
+        <v>20</v>
+      </c>
+      <c r="I1364" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1364" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="D1365" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1365" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1365" t="inlineStr">
+        <is>
+          <t>5 LBS</t>
+        </is>
+      </c>
+      <c r="G1365" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1365" t="n">
+        <v>2</v>
+      </c>
+      <c r="I1365" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1365" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="D1366" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1366" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1366" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1366" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1366" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1366" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1366" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="inlineStr">
+        <is>
+          <t>TOTALES  SUSHICORP – KN07 - KOBE MALL DEL NORTE</t>
+        </is>
+      </c>
+      <c r="F1367" t="inlineStr">
+        <is>
+          <t>3 ext.</t>
+        </is>
+      </c>
+      <c r="G1367" t="n">
+        <v>26</v>
+      </c>
+      <c r="H1367" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1368"/>
+    <row r="1369">
+      <c r="A1369" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="B1369" t="inlineStr">
+        <is>
+          <t>KN08 - NOE SAN MARINO</t>
+        </is>
+      </c>
+      <c r="C1369" t="inlineStr">
+        <is>
+          <t>NOVIEMBRE</t>
+        </is>
+      </c>
+      <c r="D1369" t="inlineStr">
+        <is>
+          <t>SALON</t>
+        </is>
+      </c>
+      <c r="E1369" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1369" t="inlineStr">
+        <is>
+          <t>50 LBS</t>
+        </is>
+      </c>
+      <c r="G1369" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1369" t="n">
+        <v>20</v>
+      </c>
+      <c r="I1369" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1369" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="D1370" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1370" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1370" t="inlineStr">
+        <is>
+          <t>5 LBS</t>
+        </is>
+      </c>
+      <c r="G1370" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1370" t="n">
+        <v>2</v>
+      </c>
+      <c r="I1370" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1370" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="D1371" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1371" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="F1371" t="inlineStr">
+        <is>
+          <t>2.5 G</t>
+        </is>
+      </c>
+      <c r="G1371" t="n">
+        <v>12</v>
+      </c>
+      <c r="H1371" t="n">
+        <v>12</v>
+      </c>
+      <c r="I1371" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1371" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="D1372" t="inlineStr">
+        <is>
+          <t>SALON</t>
+        </is>
+      </c>
+      <c r="E1372" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1372" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1372" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1372" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1372" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1372" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="D1373" t="inlineStr">
+        <is>
+          <t>SALON</t>
+        </is>
+      </c>
+      <c r="E1373" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1373" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1373" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1373" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1373" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1373" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" t="inlineStr">
+        <is>
+          <t>TOTALES  SUSHICORP – KN08 - NOE SAN MARINO</t>
+        </is>
+      </c>
+      <c r="F1374" t="inlineStr">
+        <is>
+          <t>5 ext.</t>
+        </is>
+      </c>
+      <c r="G1374" t="n">
+        <v>42</v>
+      </c>
+      <c r="H1374" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="1375"/>
+    <row r="1376">
+      <c r="A1376" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="B1376" t="inlineStr">
+        <is>
+          <t>KN09 - KOBE PLAZA TIA JOYA</t>
+        </is>
+      </c>
+      <c r="C1376" t="inlineStr">
+        <is>
+          <t>NOVIEMBRE</t>
+        </is>
+      </c>
+      <c r="D1376" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1376" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1376" t="inlineStr">
+        <is>
+          <t>50 LBS</t>
+        </is>
+      </c>
+      <c r="G1376" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1376" t="n">
+        <v>20</v>
+      </c>
+      <c r="I1376" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1376" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="D1377" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1377" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1377" t="inlineStr">
+        <is>
+          <t>5 LBS</t>
+        </is>
+      </c>
+      <c r="G1377" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1377" t="n">
+        <v>2</v>
+      </c>
+      <c r="I1377" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1377" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="D1378" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1378" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1378" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1378" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1378" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1378" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1378" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="inlineStr">
+        <is>
+          <t>TOTALES  SUSHICORP – KN09 - KOBE PLAZA TIA JOYA</t>
+        </is>
+      </c>
+      <c r="F1379" t="inlineStr">
+        <is>
+          <t>3 ext.</t>
+        </is>
+      </c>
+      <c r="G1379" t="n">
+        <v>26</v>
+      </c>
+      <c r="H1379" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1380"/>
+    <row r="1381">
+      <c r="A1381" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="B1381" t="inlineStr">
+        <is>
+          <t>KN10 - KOBE BAMBOO PLAZA VIA A LA C</t>
+        </is>
+      </c>
+      <c r="C1381" t="inlineStr">
+        <is>
+          <t>NOVIEMBRE</t>
+        </is>
+      </c>
+      <c r="D1381" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1381" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1381" t="inlineStr">
+        <is>
+          <t>50 LBS</t>
+        </is>
+      </c>
+      <c r="G1381" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1381" t="n">
+        <v>20</v>
+      </c>
+      <c r="I1381" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1381" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="D1382" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1382" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1382" t="inlineStr">
+        <is>
+          <t>5 LBS</t>
+        </is>
+      </c>
+      <c r="G1382" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1382" t="n">
+        <v>2</v>
+      </c>
+      <c r="I1382" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1382" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="D1383" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1383" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1383" t="inlineStr">
+        <is>
+          <t>5 LBS</t>
+        </is>
+      </c>
+      <c r="G1383" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1383" t="n">
+        <v>2</v>
+      </c>
+      <c r="I1383" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1383" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="inlineStr">
+        <is>
+          <t>TOTALES  SUSHICORP – KN10 - KOBE BAMBOO PLAZA VIA A LA C</t>
+        </is>
+      </c>
+      <c r="F1384" t="inlineStr">
+        <is>
+          <t>3 ext.</t>
+        </is>
+      </c>
+      <c r="G1384" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1384" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="1385"/>
+    <row r="1386">
+      <c r="A1386" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>KN11 - KOBE URDESA</t>
+        </is>
+      </c>
+      <c r="C1386" t="inlineStr">
+        <is>
+          <t>NOVIEMBRE</t>
+        </is>
+      </c>
+      <c r="D1386" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1386" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1386" t="inlineStr">
+        <is>
+          <t>50 LBS</t>
+        </is>
+      </c>
+      <c r="G1386" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1386" t="n">
+        <v>20</v>
+      </c>
+      <c r="I1386" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1386" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="D1387" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1387" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1387" t="inlineStr">
+        <is>
+          <t>20 LBS</t>
+        </is>
+      </c>
+      <c r="G1387" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1387" t="n">
+        <v>8</v>
+      </c>
+      <c r="I1387" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1387" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="D1388" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1388" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1388" t="inlineStr">
+        <is>
+          <t>20 LBS</t>
+        </is>
+      </c>
+      <c r="G1388" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1388" t="n">
+        <v>8</v>
+      </c>
+      <c r="I1388" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1388" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="D1389" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1389" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1389" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1389" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1389" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1389" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1389" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="D1390" t="inlineStr">
+        <is>
+          <t>SALON</t>
+        </is>
+      </c>
+      <c r="E1390" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1390" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1390" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1390" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1390" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1390" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="D1391" t="inlineStr">
+        <is>
+          <t>SALON</t>
+        </is>
+      </c>
+      <c r="E1391" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1391" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1391" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1391" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1391" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1391" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="D1392" t="inlineStr">
+        <is>
+          <t>SALON</t>
+        </is>
+      </c>
+      <c r="E1392" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1392" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1392" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1392" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1392" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1392" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="D1393" t="inlineStr">
+        <is>
+          <t>SALON</t>
+        </is>
+      </c>
+      <c r="E1393" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1393" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1393" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1393" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1393" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1393" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="inlineStr">
+        <is>
+          <t>TOTALES  SUSHICORP – KN11 - KOBE URDESA</t>
+        </is>
+      </c>
+      <c r="F1394" t="inlineStr">
+        <is>
+          <t>8 ext.</t>
+        </is>
+      </c>
+      <c r="G1394" t="n">
+        <v>56</v>
+      </c>
+      <c r="H1394" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1395"/>
+    <row r="1396">
+      <c r="A1396" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="B1396" t="inlineStr">
+        <is>
+          <t>KN12 - KOBE RIOC ENTRE RIOS</t>
+        </is>
+      </c>
+      <c r="C1396" t="inlineStr">
+        <is>
+          <t>DICIEMBRE</t>
+        </is>
+      </c>
+      <c r="D1396" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1396" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1396" t="inlineStr">
+        <is>
+          <t>50 LBS</t>
+        </is>
+      </c>
+      <c r="G1396" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1396" t="n">
+        <v>20</v>
+      </c>
+      <c r="I1396" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1396" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="D1397" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1397" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1397" t="inlineStr">
+        <is>
+          <t>5 LBS</t>
+        </is>
+      </c>
+      <c r="G1397" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1397" t="n">
+        <v>2</v>
+      </c>
+      <c r="I1397" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1397" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="D1398" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1398" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1398" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1398" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1398" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1398" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1398" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="inlineStr">
+        <is>
+          <t>TOTALES  SUSHICORP – KN12 - KOBE RIOC ENTRE RIOS</t>
+        </is>
+      </c>
+      <c r="F1399" t="inlineStr">
+        <is>
+          <t>3 ext.</t>
+        </is>
+      </c>
+      <c r="G1399" t="n">
+        <v>26</v>
+      </c>
+      <c r="H1399" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1400"/>
+    <row r="1401">
+      <c r="A1401" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="B1401" t="inlineStr">
+        <is>
+          <t>KN13 - KOBE RIOC CEIBOS</t>
+        </is>
+      </c>
+      <c r="C1401" t="inlineStr">
+        <is>
+          <t>DICIEMBRE</t>
+        </is>
+      </c>
+      <c r="D1401" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1401" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1401" t="inlineStr">
+        <is>
+          <t>50 LBS</t>
+        </is>
+      </c>
+      <c r="G1401" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1401" t="n">
+        <v>20</v>
+      </c>
+      <c r="I1401" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1401" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="D1402" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1402" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="F1402" t="inlineStr">
+        <is>
+          <t>5 LBS</t>
+        </is>
+      </c>
+      <c r="G1402" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1402" t="n">
+        <v>2</v>
+      </c>
+      <c r="I1402" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1402" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="D1403" t="inlineStr">
+        <is>
+          <t>COCINA</t>
+        </is>
+      </c>
+      <c r="E1403" t="inlineStr">
+        <is>
+          <t>PQS</t>
+        </is>
+      </c>
+      <c r="F1403" t="inlineStr">
+        <is>
+          <t>10 LBS</t>
+        </is>
+      </c>
+      <c r="G1403" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1403" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1403" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J1403" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" t="inlineStr">
+        <is>
+          <t>TOTALES  SUSHICORP – KN13 - KOBE RIOC CEIBOS</t>
+        </is>
+      </c>
+      <c r="F1404" t="inlineStr">
+        <is>
+          <t>3 ext.</t>
+        </is>
+      </c>
+      <c r="G1404" t="n">
+        <v>26</v>
+      </c>
+      <c r="H1404" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1405"/>
   </sheetData>
   <mergeCells count="197">
     <mergeCell ref="A5:D5"/>
@@ -45784,7 +48023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J199"/>
+  <dimension ref="A1:J212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -53720,32 +55959,548 @@
       </c>
     </row>
     <row r="199" ht="22" customHeight="1">
-      <c r="A199" s="1" t="inlineStr">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>KN01</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>KN01 - NOE MALL DEL SOL</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>FEBRERO</t>
+        </is>
+      </c>
+      <c r="E199" t="n">
+        <v>6</v>
+      </c>
+      <c r="F199" t="n">
+        <v>40</v>
+      </c>
+      <c r="G199" t="n">
+        <v>40</v>
+      </c>
+      <c r="H199" t="n">
+        <v>40</v>
+      </c>
+      <c r="I199" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J199" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>KN02</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>KN02 - NOE BOCCA SAMBO</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>FEBRERO</t>
+        </is>
+      </c>
+      <c r="E200" t="n">
+        <v>4</v>
+      </c>
+      <c r="F200" t="n">
+        <v>32</v>
+      </c>
+      <c r="G200" t="n">
+        <v>32</v>
+      </c>
+      <c r="H200" t="n">
+        <v>32</v>
+      </c>
+      <c r="I200" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J200" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>KN03</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>KN03 - KOBE PLANTA</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>FEBRERO</t>
+        </is>
+      </c>
+      <c r="E201" t="n">
+        <v>16</v>
+      </c>
+      <c r="F201" t="n">
+        <v>78</v>
+      </c>
+      <c r="G201" t="n">
+        <v>78</v>
+      </c>
+      <c r="H201" t="n">
+        <v>78</v>
+      </c>
+      <c r="I201" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J201" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>KN04</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>KN04 - KOBE SUPERCINES ORELLANA</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>MARZO</t>
+        </is>
+      </c>
+      <c r="E202" t="n">
+        <v>3</v>
+      </c>
+      <c r="F202" t="n">
+        <v>26</v>
+      </c>
+      <c r="G202" t="n">
+        <v>26</v>
+      </c>
+      <c r="H202" t="n">
+        <v>26</v>
+      </c>
+      <c r="I202" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J202" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>KN05</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>KN05 - KOBE MALL DEL SOL</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>AGOSTO</t>
+        </is>
+      </c>
+      <c r="E203" t="n">
+        <v>2</v>
+      </c>
+      <c r="F203" t="n">
+        <v>24</v>
+      </c>
+      <c r="G203" t="n">
+        <v>24</v>
+      </c>
+      <c r="H203" t="n">
+        <v>24</v>
+      </c>
+      <c r="I203" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J203" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>KN06</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>KN06 - KOBE PLAZA BATAN</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>AGOSTO</t>
+        </is>
+      </c>
+      <c r="E204" t="n">
+        <v>3</v>
+      </c>
+      <c r="F204" t="n">
+        <v>28</v>
+      </c>
+      <c r="G204" t="n">
+        <v>28</v>
+      </c>
+      <c r="H204" t="n">
+        <v>28</v>
+      </c>
+      <c r="I204" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J204" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>KN07</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>KN07 - KOBE MALL DEL NORTE</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>AGOSTO</t>
+        </is>
+      </c>
+      <c r="E205" t="n">
+        <v>3</v>
+      </c>
+      <c r="F205" t="n">
+        <v>26</v>
+      </c>
+      <c r="G205" t="n">
+        <v>26</v>
+      </c>
+      <c r="H205" t="n">
+        <v>26</v>
+      </c>
+      <c r="I205" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J205" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>KN08</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>KN08 - NOE SAN MARINO</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>NOVIEMBRE</t>
+        </is>
+      </c>
+      <c r="E206" t="n">
+        <v>5</v>
+      </c>
+      <c r="F206" t="n">
+        <v>42</v>
+      </c>
+      <c r="G206" t="n">
+        <v>42</v>
+      </c>
+      <c r="H206" t="n">
+        <v>42</v>
+      </c>
+      <c r="I206" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J206" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>KN09</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>KN09 - KOBE PLAZA TIA JOYA</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>NOVIEMBRE</t>
+        </is>
+      </c>
+      <c r="E207" t="n">
+        <v>3</v>
+      </c>
+      <c r="F207" t="n">
+        <v>26</v>
+      </c>
+      <c r="G207" t="n">
+        <v>26</v>
+      </c>
+      <c r="H207" t="n">
+        <v>26</v>
+      </c>
+      <c r="I207" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J207" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>KN10</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>KN10 - KOBE BAMBOO PLAZA VIA A LA C</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>NOVIEMBRE</t>
+        </is>
+      </c>
+      <c r="E208" t="n">
+        <v>3</v>
+      </c>
+      <c r="F208" t="n">
+        <v>24</v>
+      </c>
+      <c r="G208" t="n">
+        <v>24</v>
+      </c>
+      <c r="H208" t="n">
+        <v>24</v>
+      </c>
+      <c r="I208" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J208" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>KN11</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>KN11 - KOBE URDESA</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>NOVIEMBRE</t>
+        </is>
+      </c>
+      <c r="E209" t="n">
+        <v>8</v>
+      </c>
+      <c r="F209" t="n">
+        <v>56</v>
+      </c>
+      <c r="G209" t="n">
+        <v>56</v>
+      </c>
+      <c r="H209" t="n">
+        <v>56</v>
+      </c>
+      <c r="I209" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J209" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>KN12</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>KN12 - KOBE RIOC ENTRE RIOS</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>DICIEMBRE</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>3</v>
+      </c>
+      <c r="F210" t="n">
+        <v>26</v>
+      </c>
+      <c r="G210" t="n">
+        <v>26</v>
+      </c>
+      <c r="H210" t="n">
+        <v>26</v>
+      </c>
+      <c r="I210" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J210" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>KN13</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>SUSHICORP</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>KN13 - KOBE RIOC CEIBOS</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>DICIEMBRE</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>3</v>
+      </c>
+      <c r="F211" t="n">
+        <v>26</v>
+      </c>
+      <c r="G211" t="n">
+        <v>26</v>
+      </c>
+      <c r="H211" t="n">
+        <v>26</v>
+      </c>
+      <c r="I211" t="n">
+        <v>2024</v>
+      </c>
+      <c r="J211" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
         <is>
           <t>GRAN TOTAL</t>
         </is>
       </c>
-      <c r="B199" s="1" t="inlineStr"/>
-      <c r="C199" s="1" t="inlineStr">
-        <is>
-          <t>197 LOCALES</t>
-        </is>
-      </c>
-      <c r="D199" s="1" t="inlineStr"/>
-      <c r="E199" s="1" t="n">
-        <v>906</v>
-      </c>
-      <c r="F199" s="15" t="n">
-        <v>7072.3</v>
-      </c>
-      <c r="G199" s="15" t="n">
-        <v>20133.2</v>
-      </c>
-      <c r="H199" s="15" t="n">
-        <v>20108.2</v>
-      </c>
-      <c r="I199" s="1" t="inlineStr"/>
-      <c r="J199" s="1" t="inlineStr"/>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>210 LOCALES</t>
+        </is>
+      </c>
+      <c r="E212" t="n">
+        <v>968</v>
+      </c>
+      <c r="F212" t="n">
+        <v>7526.3</v>
+      </c>
+      <c r="G212" t="n">
+        <v>20587.2</v>
+      </c>
+      <c r="H212" t="n">
+        <v>20562.2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Separate SUSHICORP into independent Excel file
- BASE_DATOS_KFC.xlsx: removed 13 KN locales (now 197 locales, KFC group only)
- BASE_DATOS_SUSHICORP.xlsx: new file with 13 SUSHICORP locals (KN01-KN13)
  Same structure: RESUMEN_LOCALES + DETALLE sheets
- separar_sushicorp.py: script used to perform the split

https://claude.ai/code/session_017rdRDT2VUBvb4GkrdojQaa
</commit_message>
<xml_diff>
--- a/BASE_DATOS_KFC.xlsx
+++ b/BASE_DATOS_KFC.xlsx
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1405"/>
+  <dimension ref="A1:J1317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -45573,2246 +45573,7 @@
       <c r="I1317" s="4" t="inlineStr"/>
       <c r="J1317" s="4" t="inlineStr"/>
     </row>
-    <row r="1318" ht="8" customHeight="1">
-      <c r="A1318" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1318" t="inlineStr">
-        <is>
-          <t>KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1318" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1318" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1318" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1318" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1318" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1318" t="n">
-        <v>20</v>
-      </c>
-      <c r="I1318" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1318" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1319">
-      <c r="D1319" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1319" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1319" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1319" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1319" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1319" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1319" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1320">
-      <c r="D1320" t="inlineStr">
-        <is>
-          <t>OFICINA</t>
-        </is>
-      </c>
-      <c r="E1320" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1320" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1320" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1320" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1320" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1320" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1321">
-      <c r="D1321" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1321" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1321" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1321" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1321" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1321" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1321" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1322">
-      <c r="D1322" t="inlineStr">
-        <is>
-          <t>GABINETE ENTRADA</t>
-        </is>
-      </c>
-      <c r="E1322" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1322" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1322" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1322" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1322" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1322" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1323">
-      <c r="D1323" t="inlineStr">
-        <is>
-          <t>BODEGA</t>
-        </is>
-      </c>
-      <c r="E1323" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1323" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1323" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1323" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1323" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1323" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1324">
-      <c r="A1324" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="F1324" t="inlineStr">
-        <is>
-          <t>6 ext.</t>
-        </is>
-      </c>
-      <c r="G1324" t="n">
-        <v>40</v>
-      </c>
-      <c r="H1324" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="1325"/>
-    <row r="1326">
-      <c r="A1326" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1326" t="inlineStr">
-        <is>
-          <t>KN02 - NOE BOCCA SAMBO</t>
-        </is>
-      </c>
-      <c r="C1326" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1326" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1326" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1326" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1326" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1326" t="n">
-        <v>20</v>
-      </c>
-      <c r="I1326" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1326" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1327">
-      <c r="D1327" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1327" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1327" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1327" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1327" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1327" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1327" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1328">
-      <c r="D1328" t="inlineStr">
-        <is>
-          <t>BODEGA</t>
-        </is>
-      </c>
-      <c r="E1328" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1328" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1328" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1328" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1328" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1328" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1329">
-      <c r="D1329" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1329" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1329" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1329" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1329" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1329" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1329" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1330">
-      <c r="A1330" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN02 - NOE BOCCA SAMBO</t>
-        </is>
-      </c>
-      <c r="F1330" t="inlineStr">
-        <is>
-          <t>4 ext.</t>
-        </is>
-      </c>
-      <c r="G1330" t="n">
-        <v>32</v>
-      </c>
-      <c r="H1330" t="n">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="1331"/>
-    <row r="1332">
-      <c r="A1332" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1332" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1332" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1332" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1332" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1332" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1332" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1332" t="n">
-        <v>20</v>
-      </c>
-      <c r="I1332" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1332" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1333">
-      <c r="D1333" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1333" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1333" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1333" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1333" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1333" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1333" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1334">
-      <c r="D1334" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1334" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1334" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1334" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1334" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1334" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1334" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1335">
-      <c r="D1335" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1335" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1335" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1335" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1335" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1335" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1335" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1336">
-      <c r="D1336" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1336" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1336" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1336" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1336" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1336" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1336" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1337">
-      <c r="D1337" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1337" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1337" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1337" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1337" t="n">
-        <v>2</v>
-      </c>
-      <c r="I1337" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1337" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1338">
-      <c r="D1338" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1338" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1338" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1338" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1338" t="n">
-        <v>2</v>
-      </c>
-      <c r="I1338" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1338" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1339">
-      <c r="D1339" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1339" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1339" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1339" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1339" t="n">
-        <v>2</v>
-      </c>
-      <c r="I1339" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1339" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1340">
-      <c r="D1340" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1340" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1340" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1340" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1340" t="n">
-        <v>2</v>
-      </c>
-      <c r="I1340" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1340" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1341">
-      <c r="D1341" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1341" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1341" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1341" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1341" t="n">
-        <v>2</v>
-      </c>
-      <c r="I1341" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1341" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1342">
-      <c r="D1342" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1342" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1342" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1342" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1342" t="n">
-        <v>8</v>
-      </c>
-      <c r="I1342" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1342" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1343">
-      <c r="D1343" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1343" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1343" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1343" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1343" t="n">
-        <v>8</v>
-      </c>
-      <c r="I1343" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1343" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1344">
-      <c r="D1344" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1344" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1344" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1344" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1344" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1344" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1344" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1345">
-      <c r="D1345" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1345" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1345" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1345" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1345" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1345" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1345" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1346">
-      <c r="D1346" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1346" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1346" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1346" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1346" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1346" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1346" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1347">
-      <c r="D1347" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1347" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1347" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1347" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1347" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1347" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1347" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1348">
-      <c r="A1348" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="F1348" t="inlineStr">
-        <is>
-          <t>16 ext.</t>
-        </is>
-      </c>
-      <c r="G1348" t="n">
-        <v>78</v>
-      </c>
-      <c r="H1348" t="n">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="1349"/>
-    <row r="1350">
-      <c r="A1350" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1350" t="inlineStr">
-        <is>
-          <t>KN04 - KOBE SUPERCINES ORELLANA</t>
-        </is>
-      </c>
-      <c r="C1350" t="inlineStr">
-        <is>
-          <t>MARZO</t>
-        </is>
-      </c>
-      <c r="D1350" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1350" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1350" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1350" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1350" t="n">
-        <v>20</v>
-      </c>
-      <c r="I1350" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1350" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1351">
-      <c r="D1351" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1351" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1351" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1351" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1351" t="n">
-        <v>2</v>
-      </c>
-      <c r="I1351" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1351" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1352">
-      <c r="D1352" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1352" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1352" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1352" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1352" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1352" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1352" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1353">
-      <c r="A1353" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN04 - KOBE SUPERCINES ORELLANA</t>
-        </is>
-      </c>
-      <c r="F1353" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1353" t="n">
-        <v>26</v>
-      </c>
-      <c r="H1353" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="1354"/>
-    <row r="1355">
-      <c r="A1355" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1355" t="inlineStr">
-        <is>
-          <t>KN05 - KOBE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1355" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1355" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1355" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1355" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1355" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1355" t="n">
-        <v>20</v>
-      </c>
-      <c r="I1355" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1355" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1356">
-      <c r="D1356" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1356" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1356" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1356" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1356" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1356" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1356" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1357">
-      <c r="A1357" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN05 - KOBE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="F1357" t="inlineStr">
-        <is>
-          <t>2 ext.</t>
-        </is>
-      </c>
-      <c r="G1357" t="n">
-        <v>24</v>
-      </c>
-      <c r="H1357" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="1358"/>
-    <row r="1359">
-      <c r="A1359" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1359" t="inlineStr">
-        <is>
-          <t>KN06 - KOBE PLAZA BATAN</t>
-        </is>
-      </c>
-      <c r="C1359" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1359" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1359" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1359" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1359" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1359" t="n">
-        <v>20</v>
-      </c>
-      <c r="I1359" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1359" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1360">
-      <c r="D1360" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1360" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1360" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1360" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1360" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1360" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1360" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1361">
-      <c r="D1361" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1361" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1361" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1361" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1361" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1361" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1361" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1362">
-      <c r="A1362" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN06 - KOBE PLAZA BATAN</t>
-        </is>
-      </c>
-      <c r="F1362" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1362" t="n">
-        <v>28</v>
-      </c>
-      <c r="H1362" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="1363"/>
-    <row r="1364">
-      <c r="A1364" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1364" t="inlineStr">
-        <is>
-          <t>KN07 - KOBE MALL DEL NORTE</t>
-        </is>
-      </c>
-      <c r="C1364" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1364" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1364" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1364" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1364" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1364" t="n">
-        <v>20</v>
-      </c>
-      <c r="I1364" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1364" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1365">
-      <c r="D1365" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1365" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1365" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1365" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1365" t="n">
-        <v>2</v>
-      </c>
-      <c r="I1365" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1365" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1366">
-      <c r="D1366" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1366" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1366" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1366" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1366" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1366" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1366" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1367">
-      <c r="A1367" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN07 - KOBE MALL DEL NORTE</t>
-        </is>
-      </c>
-      <c r="F1367" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1367" t="n">
-        <v>26</v>
-      </c>
-      <c r="H1367" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="1368"/>
-    <row r="1369">
-      <c r="A1369" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1369" t="inlineStr">
-        <is>
-          <t>KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="C1369" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1369" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1369" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1369" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1369" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1369" t="n">
-        <v>20</v>
-      </c>
-      <c r="I1369" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1369" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1370">
-      <c r="D1370" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1370" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1370" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1370" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1370" t="n">
-        <v>2</v>
-      </c>
-      <c r="I1370" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1370" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1371">
-      <c r="D1371" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1371" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="F1371" t="inlineStr">
-        <is>
-          <t>2.5 G</t>
-        </is>
-      </c>
-      <c r="G1371" t="n">
-        <v>12</v>
-      </c>
-      <c r="H1371" t="n">
-        <v>12</v>
-      </c>
-      <c r="I1371" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1371" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1372">
-      <c r="D1372" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1372" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1372" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1372" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1372" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1372" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1372" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1373">
-      <c r="D1373" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1373" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1373" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1373" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1373" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1373" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1373" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1374">
-      <c r="A1374" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="F1374" t="inlineStr">
-        <is>
-          <t>5 ext.</t>
-        </is>
-      </c>
-      <c r="G1374" t="n">
-        <v>42</v>
-      </c>
-      <c r="H1374" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="1375"/>
-    <row r="1376">
-      <c r="A1376" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1376" t="inlineStr">
-        <is>
-          <t>KN09 - KOBE PLAZA TIA JOYA</t>
-        </is>
-      </c>
-      <c r="C1376" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1376" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1376" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1376" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1376" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1376" t="n">
-        <v>20</v>
-      </c>
-      <c r="I1376" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1376" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1377">
-      <c r="D1377" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1377" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1377" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1377" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1377" t="n">
-        <v>2</v>
-      </c>
-      <c r="I1377" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1377" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1378">
-      <c r="D1378" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1378" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1378" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1378" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1378" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1378" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1378" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1379">
-      <c r="A1379" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN09 - KOBE PLAZA TIA JOYA</t>
-        </is>
-      </c>
-      <c r="F1379" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1379" t="n">
-        <v>26</v>
-      </c>
-      <c r="H1379" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="1380"/>
-    <row r="1381">
-      <c r="A1381" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1381" t="inlineStr">
-        <is>
-          <t>KN10 - KOBE BAMBOO PLAZA VIA A LA C</t>
-        </is>
-      </c>
-      <c r="C1381" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1381" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1381" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1381" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1381" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1381" t="n">
-        <v>20</v>
-      </c>
-      <c r="I1381" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1381" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1382">
-      <c r="D1382" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1382" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1382" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1382" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1382" t="n">
-        <v>2</v>
-      </c>
-      <c r="I1382" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1382" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1383">
-      <c r="D1383" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1383" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1383" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1383" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1383" t="n">
-        <v>2</v>
-      </c>
-      <c r="I1383" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1383" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1384">
-      <c r="A1384" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN10 - KOBE BAMBOO PLAZA VIA A LA C</t>
-        </is>
-      </c>
-      <c r="F1384" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1384" t="n">
-        <v>24</v>
-      </c>
-      <c r="H1384" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="1385"/>
-    <row r="1386">
-      <c r="A1386" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1386" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1386" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1386" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1386" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1386" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1386" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1386" t="n">
-        <v>20</v>
-      </c>
-      <c r="I1386" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1386" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1387">
-      <c r="D1387" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1387" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1387" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1387" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1387" t="n">
-        <v>8</v>
-      </c>
-      <c r="I1387" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1387" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1388">
-      <c r="D1388" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1388" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1388" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1388" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1388" t="n">
-        <v>8</v>
-      </c>
-      <c r="I1388" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1388" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1389">
-      <c r="D1389" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1389" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1389" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1389" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1389" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1389" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1389" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1390">
-      <c r="D1390" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1390" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1390" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1390" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1390" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1390" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1390" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1391">
-      <c r="D1391" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1391" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1391" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1391" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1391" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1391" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1391" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1392">
-      <c r="D1392" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1392" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1392" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1392" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1392" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1392" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1392" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1393">
-      <c r="D1393" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1393" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1393" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1393" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1393" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1393" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1393" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1394">
-      <c r="A1394" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="F1394" t="inlineStr">
-        <is>
-          <t>8 ext.</t>
-        </is>
-      </c>
-      <c r="G1394" t="n">
-        <v>56</v>
-      </c>
-      <c r="H1394" t="n">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="1395"/>
-    <row r="1396">
-      <c r="A1396" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1396" t="inlineStr">
-        <is>
-          <t>KN12 - KOBE RIOC ENTRE RIOS</t>
-        </is>
-      </c>
-      <c r="C1396" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1396" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1396" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1396" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1396" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1396" t="n">
-        <v>20</v>
-      </c>
-      <c r="I1396" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1396" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1397">
-      <c r="D1397" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1397" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1397" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1397" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1397" t="n">
-        <v>2</v>
-      </c>
-      <c r="I1397" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1397" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1398">
-      <c r="D1398" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1398" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1398" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1398" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1398" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1398" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1398" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1399">
-      <c r="A1399" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN12 - KOBE RIOC ENTRE RIOS</t>
-        </is>
-      </c>
-      <c r="F1399" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1399" t="n">
-        <v>26</v>
-      </c>
-      <c r="H1399" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="1400"/>
-    <row r="1401">
-      <c r="A1401" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1401" t="inlineStr">
-        <is>
-          <t>KN13 - KOBE RIOC CEIBOS</t>
-        </is>
-      </c>
-      <c r="C1401" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1401" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1401" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1401" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1401" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1401" t="n">
-        <v>20</v>
-      </c>
-      <c r="I1401" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1401" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1402">
-      <c r="D1402" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1402" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1402" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1402" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1402" t="n">
-        <v>2</v>
-      </c>
-      <c r="I1402" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1402" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1403">
-      <c r="D1403" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1403" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1403" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1403" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1403" t="n">
-        <v>4</v>
-      </c>
-      <c r="I1403" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1403" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1404">
-      <c r="A1404" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN13 - KOBE RIOC CEIBOS</t>
-        </is>
-      </c>
-      <c r="F1404" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1404" t="n">
-        <v>26</v>
-      </c>
-      <c r="H1404" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="1405"/>
+    <row r="1318" ht="8" customHeight="1"/>
   </sheetData>
   <mergeCells count="197">
     <mergeCell ref="A5:D5"/>
@@ -48023,7 +45784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J212"/>
+  <dimension ref="A1:J199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -55961,545 +53722,25 @@
     <row r="199" ht="22" customHeight="1">
       <c r="A199" t="inlineStr">
         <is>
-          <t>KN01</t>
-        </is>
-      </c>
-      <c r="B199" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
+          <t>GRAN TOTAL</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="D199" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
+          <t>197 LOCALES</t>
         </is>
       </c>
       <c r="E199" t="n">
-        <v>6</v>
+        <v>906</v>
       </c>
       <c r="F199" t="n">
-        <v>40</v>
+        <v>7072.3</v>
       </c>
       <c r="G199" t="n">
-        <v>40</v>
+        <v>20133.2</v>
       </c>
       <c r="H199" t="n">
-        <v>40</v>
-      </c>
-      <c r="I199" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J199" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>KN02</t>
-        </is>
-      </c>
-      <c r="B200" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C200" t="inlineStr">
-        <is>
-          <t>KN02 - NOE BOCCA SAMBO</t>
-        </is>
-      </c>
-      <c r="D200" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="E200" t="n">
-        <v>4</v>
-      </c>
-      <c r="F200" t="n">
-        <v>32</v>
-      </c>
-      <c r="G200" t="n">
-        <v>32</v>
-      </c>
-      <c r="H200" t="n">
-        <v>32</v>
-      </c>
-      <c r="I200" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J200" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>KN03</t>
-        </is>
-      </c>
-      <c r="B201" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C201" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="D201" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="E201" t="n">
-        <v>16</v>
-      </c>
-      <c r="F201" t="n">
-        <v>78</v>
-      </c>
-      <c r="G201" t="n">
-        <v>78</v>
-      </c>
-      <c r="H201" t="n">
-        <v>78</v>
-      </c>
-      <c r="I201" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J201" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>KN04</t>
-        </is>
-      </c>
-      <c r="B202" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C202" t="inlineStr">
-        <is>
-          <t>KN04 - KOBE SUPERCINES ORELLANA</t>
-        </is>
-      </c>
-      <c r="D202" t="inlineStr">
-        <is>
-          <t>MARZO</t>
-        </is>
-      </c>
-      <c r="E202" t="n">
-        <v>3</v>
-      </c>
-      <c r="F202" t="n">
-        <v>26</v>
-      </c>
-      <c r="G202" t="n">
-        <v>26</v>
-      </c>
-      <c r="H202" t="n">
-        <v>26</v>
-      </c>
-      <c r="I202" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J202" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>KN05</t>
-        </is>
-      </c>
-      <c r="B203" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C203" t="inlineStr">
-        <is>
-          <t>KN05 - KOBE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="D203" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="E203" t="n">
-        <v>2</v>
-      </c>
-      <c r="F203" t="n">
-        <v>24</v>
-      </c>
-      <c r="G203" t="n">
-        <v>24</v>
-      </c>
-      <c r="H203" t="n">
-        <v>24</v>
-      </c>
-      <c r="I203" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J203" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="inlineStr">
-        <is>
-          <t>KN06</t>
-        </is>
-      </c>
-      <c r="B204" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C204" t="inlineStr">
-        <is>
-          <t>KN06 - KOBE PLAZA BATAN</t>
-        </is>
-      </c>
-      <c r="D204" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="E204" t="n">
-        <v>3</v>
-      </c>
-      <c r="F204" t="n">
-        <v>28</v>
-      </c>
-      <c r="G204" t="n">
-        <v>28</v>
-      </c>
-      <c r="H204" t="n">
-        <v>28</v>
-      </c>
-      <c r="I204" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J204" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="inlineStr">
-        <is>
-          <t>KN07</t>
-        </is>
-      </c>
-      <c r="B205" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C205" t="inlineStr">
-        <is>
-          <t>KN07 - KOBE MALL DEL NORTE</t>
-        </is>
-      </c>
-      <c r="D205" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="E205" t="n">
-        <v>3</v>
-      </c>
-      <c r="F205" t="n">
-        <v>26</v>
-      </c>
-      <c r="G205" t="n">
-        <v>26</v>
-      </c>
-      <c r="H205" t="n">
-        <v>26</v>
-      </c>
-      <c r="I205" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J205" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>KN08</t>
-        </is>
-      </c>
-      <c r="B206" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C206" t="inlineStr">
-        <is>
-          <t>KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="D206" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="E206" t="n">
-        <v>5</v>
-      </c>
-      <c r="F206" t="n">
-        <v>42</v>
-      </c>
-      <c r="G206" t="n">
-        <v>42</v>
-      </c>
-      <c r="H206" t="n">
-        <v>42</v>
-      </c>
-      <c r="I206" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J206" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>KN09</t>
-        </is>
-      </c>
-      <c r="B207" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C207" t="inlineStr">
-        <is>
-          <t>KN09 - KOBE PLAZA TIA JOYA</t>
-        </is>
-      </c>
-      <c r="D207" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="E207" t="n">
-        <v>3</v>
-      </c>
-      <c r="F207" t="n">
-        <v>26</v>
-      </c>
-      <c r="G207" t="n">
-        <v>26</v>
-      </c>
-      <c r="H207" t="n">
-        <v>26</v>
-      </c>
-      <c r="I207" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J207" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>KN10</t>
-        </is>
-      </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C208" t="inlineStr">
-        <is>
-          <t>KN10 - KOBE BAMBOO PLAZA VIA A LA C</t>
-        </is>
-      </c>
-      <c r="D208" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="E208" t="n">
-        <v>3</v>
-      </c>
-      <c r="F208" t="n">
-        <v>24</v>
-      </c>
-      <c r="G208" t="n">
-        <v>24</v>
-      </c>
-      <c r="H208" t="n">
-        <v>24</v>
-      </c>
-      <c r="I208" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J208" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>KN11</t>
-        </is>
-      </c>
-      <c r="B209" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C209" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="D209" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="E209" t="n">
-        <v>8</v>
-      </c>
-      <c r="F209" t="n">
-        <v>56</v>
-      </c>
-      <c r="G209" t="n">
-        <v>56</v>
-      </c>
-      <c r="H209" t="n">
-        <v>56</v>
-      </c>
-      <c r="I209" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J209" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="inlineStr">
-        <is>
-          <t>KN12</t>
-        </is>
-      </c>
-      <c r="B210" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C210" t="inlineStr">
-        <is>
-          <t>KN12 - KOBE RIOC ENTRE RIOS</t>
-        </is>
-      </c>
-      <c r="D210" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="E210" t="n">
-        <v>3</v>
-      </c>
-      <c r="F210" t="n">
-        <v>26</v>
-      </c>
-      <c r="G210" t="n">
-        <v>26</v>
-      </c>
-      <c r="H210" t="n">
-        <v>26</v>
-      </c>
-      <c r="I210" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J210" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>KN13</t>
-        </is>
-      </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C211" t="inlineStr">
-        <is>
-          <t>KN13 - KOBE RIOC CEIBOS</t>
-        </is>
-      </c>
-      <c r="D211" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="E211" t="n">
-        <v>3</v>
-      </c>
-      <c r="F211" t="n">
-        <v>26</v>
-      </c>
-      <c r="G211" t="n">
-        <v>26</v>
-      </c>
-      <c r="H211" t="n">
-        <v>26</v>
-      </c>
-      <c r="I211" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J211" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>GRAN TOTAL</t>
-        </is>
-      </c>
-      <c r="C212" t="inlineStr">
-        <is>
-          <t>210 LOCALES</t>
-        </is>
-      </c>
-      <c r="E212" t="n">
-        <v>968</v>
-      </c>
-      <c r="F212" t="n">
-        <v>7526.3</v>
-      </c>
-      <c r="G212" t="n">
-        <v>20587.2</v>
-      </c>
-      <c r="H212" t="n">
-        <v>20562.2</v>
+        <v>20108.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix data inconsistency: KN008 extinguisher type "K" → "TIPO K", capacity "2.5 G" → "2.5 GLS"
Fixed in both DETALLE (row 1368) and NOVIEMBRE (row 171) sheets.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFXpAjF8wqo1CCwLa1Q85Z
</commit_message>
<xml_diff>
--- a/BASE_DATOS_KFC.xlsx
+++ b/BASE_DATOS_KFC.xlsx
@@ -45383,6 +45383,7 @@
         <v>94</v>
       </c>
     </row>
+    <row r="1322"/>
     <row r="1323">
       <c r="A1323" t="inlineStr">
         <is>
@@ -45532,6 +45533,7 @@
         <v>74.40000000000001</v>
       </c>
     </row>
+    <row r="1328"/>
     <row r="1329">
       <c r="A1329" t="inlineStr">
         <is>
@@ -46029,6 +46031,7 @@
         <v>181.9</v>
       </c>
     </row>
+    <row r="1346"/>
     <row r="1347">
       <c r="A1347" t="inlineStr">
         <is>
@@ -46149,6 +46152,7 @@
         <v>59.3</v>
       </c>
     </row>
+    <row r="1351"/>
     <row r="1352">
       <c r="A1352" t="inlineStr">
         <is>
@@ -46240,6 +46244,7 @@
         <v>54.8</v>
       </c>
     </row>
+    <row r="1355"/>
     <row r="1356">
       <c r="A1356" t="inlineStr">
         <is>
@@ -46360,6 +46365,7 @@
         <v>64.59999999999999</v>
       </c>
     </row>
+    <row r="1360"/>
     <row r="1361">
       <c r="A1361" t="inlineStr">
         <is>
@@ -46480,6 +46486,7 @@
         <v>59.3</v>
       </c>
     </row>
+    <row r="1365"/>
     <row r="1366">
       <c r="A1366" t="inlineStr">
         <is>
@@ -46561,12 +46568,12 @@
       </c>
       <c r="E1368" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>TIPO K</t>
         </is>
       </c>
       <c r="F1368" t="inlineStr">
         <is>
-          <t>2.5 G</t>
+          <t>2.5 GLS</t>
         </is>
       </c>
       <c r="G1368" t="n">
@@ -46658,6 +46665,7 @@
         <v>81.09999999999999</v>
       </c>
     </row>
+    <row r="1372"/>
     <row r="1373">
       <c r="A1373" t="inlineStr">
         <is>
@@ -46778,6 +46786,7 @@
         <v>59.3</v>
       </c>
     </row>
+    <row r="1377"/>
     <row r="1378">
       <c r="A1378" t="inlineStr">
         <is>
@@ -46898,6 +46907,7 @@
         <v>54</v>
       </c>
     </row>
+    <row r="1382"/>
     <row r="1383">
       <c r="A1383" t="inlineStr">
         <is>
@@ -47163,6 +47173,7 @@
         <v>133.2</v>
       </c>
     </row>
+    <row r="1392"/>
     <row r="1393">
       <c r="A1393" t="inlineStr">
         <is>
@@ -47283,6 +47294,7 @@
         <v>59.3</v>
       </c>
     </row>
+    <row r="1397"/>
     <row r="1398">
       <c r="A1398" t="inlineStr">
         <is>
@@ -47873,6 +47885,7 @@
         <v>63.8</v>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -47930,6 +47943,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -47987,6 +48001,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -48313,6 +48328,7 @@
         <v>108.3</v>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
@@ -48419,6 +48435,7 @@
         <v>13.9</v>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
@@ -48851,6 +48868,7 @@
         <v>102.2</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -49001,6 +49019,7 @@
         <v>19.2</v>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -49107,6 +49126,7 @@
         <v>14.3</v>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -49301,6 +49321,7 @@
         <v>63.8</v>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
@@ -49592,6 +49613,7 @@
         <v>97.7</v>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
@@ -49830,6 +49852,7 @@
         <v>72.8</v>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
@@ -50156,6 +50179,7 @@
         <v>124.7</v>
       </c>
     </row>
+    <row r="50"/>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
@@ -50790,6 +50814,7 @@
         <v>241.2</v>
       </c>
     </row>
+    <row r="66"/>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
@@ -50984,6 +51009,7 @@
         <v>63.8</v>
       </c>
     </row>
+    <row r="72"/>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
@@ -51442,6 +51468,7 @@
         <v>152</v>
       </c>
     </row>
+    <row r="84"/>
     <row r="85">
       <c r="A85" s="17" t="inlineStr">
         <is>
@@ -51742,6 +51769,7 @@
         <v>162.6</v>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -51848,6 +51876,7 @@
         <v>19.6</v>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -52042,6 +52071,7 @@
         <v>63.8</v>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
@@ -52236,6 +52266,7 @@
         <v>162.6</v>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
@@ -52430,6 +52461,7 @@
         <v>162.6</v>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
@@ -52624,6 +52656,7 @@
         <v>162.6</v>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
@@ -52906,6 +52939,7 @@
         <v>167.1</v>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
@@ -53100,6 +53134,7 @@
         <v>69.09999999999999</v>
       </c>
     </row>
+    <row r="49"/>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
@@ -53382,6 +53417,7 @@
         <v>167.9</v>
       </c>
     </row>
+    <row r="57"/>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
@@ -53620,6 +53656,7 @@
         <v>83.40000000000001</v>
       </c>
     </row>
+    <row r="64"/>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
@@ -53858,6 +53895,7 @@
         <v>81.8</v>
       </c>
     </row>
+    <row r="71"/>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
@@ -54188,6 +54226,7 @@
         <v>221.4</v>
       </c>
     </row>
+    <row r="81"/>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
@@ -54646,6 +54685,7 @@
         <v>244.7</v>
       </c>
     </row>
+    <row r="93"/>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
@@ -55060,6 +55100,7 @@
         <v>206.3</v>
       </c>
     </row>
+    <row r="104"/>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
@@ -55342,6 +55383,7 @@
         <v>167.1</v>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
@@ -55756,6 +55798,7 @@
         <v>240.2</v>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
@@ -55950,6 +55993,7 @@
         <v>72.8</v>
       </c>
     </row>
+    <row r="129"/>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
@@ -56232,6 +56276,7 @@
         <v>167.1</v>
       </c>
     </row>
+    <row r="137"/>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
@@ -56426,6 +56471,7 @@
         <v>172.4</v>
       </c>
     </row>
+    <row r="143"/>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
@@ -56532,6 +56578,7 @@
         <v>19.6</v>
       </c>
     </row>
+    <row r="147"/>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
@@ -56638,6 +56685,7 @@
         <v>19.6</v>
       </c>
     </row>
+    <row r="151"/>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
@@ -56744,6 +56792,7 @@
         <v>19.6</v>
       </c>
     </row>
+    <row r="155"/>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
@@ -56850,6 +56899,7 @@
         <v>19.6</v>
       </c>
     </row>
+    <row r="159"/>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
@@ -56912,6 +56962,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="162"/>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
@@ -56974,6 +57025,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="165"/>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
@@ -57036,6 +57088,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="168"/>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
@@ -57117,12 +57170,12 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>TIPO K</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>2.5 G</t>
+          <t>2.5 GLS</t>
         </is>
       </c>
       <c r="G171" t="n">
@@ -57214,6 +57267,7 @@
         <v>81.09999999999999</v>
       </c>
     </row>
+    <row r="175"/>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
@@ -57334,6 +57388,7 @@
         <v>59.3</v>
       </c>
     </row>
+    <row r="180"/>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
@@ -57454,6 +57509,7 @@
         <v>54</v>
       </c>
     </row>
+    <row r="185"/>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
@@ -57719,6 +57775,7 @@
         <v>133.2</v>
       </c>
     </row>
+    <row r="195"/>
     <row r="196">
       <c r="A196" s="17" t="inlineStr">
         <is>
@@ -58019,6 +58076,7 @@
         <v>78.90000000000001</v>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -58213,6 +58271,7 @@
         <v>72.8</v>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -58451,6 +58510,7 @@
         <v>178.1</v>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
@@ -58689,6 +58749,7 @@
         <v>83.40000000000001</v>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
@@ -59191,6 +59252,7 @@
         <v>270.4</v>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
@@ -59781,6 +59843,7 @@
         <v>298.2</v>
       </c>
     </row>
+    <row r="55"/>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
@@ -60151,6 +60214,7 @@
         <v>205.5</v>
       </c>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
@@ -60345,6 +60409,7 @@
         <v>158.1</v>
       </c>
     </row>
+    <row r="71"/>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
@@ -60495,6 +60560,7 @@
         <v>24.1</v>
       </c>
     </row>
+    <row r="76"/>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
@@ -60557,6 +60623,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="79"/>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
@@ -60677,6 +60744,7 @@
         <v>59.3</v>
       </c>
     </row>
+    <row r="84"/>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
@@ -60797,6 +60865,7 @@
         <v>59.3</v>
       </c>
     </row>
+    <row r="89"/>
     <row r="90">
       <c r="A90" s="17" t="inlineStr">
         <is>
@@ -61053,6 +61122,7 @@
         <v>63.8</v>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -61291,6 +61361,7 @@
         <v>83.40000000000001</v>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -61661,6 +61732,7 @@
         <v>167.6</v>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
@@ -61899,6 +61971,7 @@
         <v>105.9</v>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
@@ -62049,6 +62122,7 @@
         <v>64.59999999999999</v>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
@@ -62375,6 +62449,7 @@
         <v>145.9</v>
       </c>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
@@ -62701,6 +62776,7 @@
         <v>192</v>
       </c>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
@@ -62895,6 +62971,7 @@
         <v>73.59999999999999</v>
       </c>
     </row>
+    <row r="59"/>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
@@ -63089,6 +63166,7 @@
         <v>74.40000000000001</v>
       </c>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
@@ -63459,6 +63537,7 @@
         <v>163.9</v>
       </c>
     </row>
+    <row r="75"/>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
@@ -63785,6 +63864,7 @@
         <v>93.2</v>
       </c>
     </row>
+    <row r="84"/>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
@@ -63979,6 +64059,7 @@
         <v>96.90000000000001</v>
       </c>
     </row>
+    <row r="90"/>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
@@ -64173,6 +64254,7 @@
         <v>105.9</v>
       </c>
     </row>
+    <row r="96"/>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
@@ -64455,6 +64537,7 @@
         <v>172.8</v>
       </c>
     </row>
+    <row r="104"/>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
@@ -64649,6 +64732,7 @@
         <v>167.9</v>
       </c>
     </row>
+    <row r="110"/>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
@@ -64843,6 +64927,7 @@
         <v>101.4</v>
       </c>
     </row>
+    <row r="116"/>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
@@ -65169,6 +65254,7 @@
         <v>192</v>
       </c>
     </row>
+    <row r="125"/>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
@@ -65583,6 +65669,7 @@
         <v>206.3</v>
       </c>
     </row>
+    <row r="136"/>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
@@ -65777,6 +65864,7 @@
         <v>101.4</v>
       </c>
     </row>
+    <row r="142"/>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
@@ -66191,6 +66279,7 @@
         <v>162.6</v>
       </c>
     </row>
+    <row r="153"/>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
@@ -66473,6 +66562,7 @@
         <v>172.4</v>
       </c>
     </row>
+    <row r="161"/>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
@@ -66667,6 +66757,7 @@
         <v>63.8</v>
       </c>
     </row>
+    <row r="167"/>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
@@ -66773,6 +66864,7 @@
         <v>19.6</v>
       </c>
     </row>
+    <row r="171"/>
     <row r="172">
       <c r="A172" s="17" t="inlineStr">
         <is>
@@ -67073,6 +67165,7 @@
         <v>72.8</v>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -67179,6 +67272,7 @@
         <v>18.8</v>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -67241,6 +67335,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -67303,6 +67398,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
@@ -67409,6 +67505,7 @@
         <v>19.6</v>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
@@ -67515,6 +67612,7 @@
         <v>14.3</v>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
@@ -67621,6 +67719,7 @@
         <v>19.6</v>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
@@ -67771,6 +67870,7 @@
         <v>19.2</v>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
@@ -67921,6 +68021,7 @@
         <v>64.59999999999999</v>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
@@ -68203,6 +68304,7 @@
         <v>172</v>
       </c>
     </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
@@ -68573,6 +68675,7 @@
         <v>107.9</v>
       </c>
     </row>
+    <row r="57"/>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
@@ -69075,6 +69178,7 @@
         <v>167.1</v>
       </c>
     </row>
+    <row r="70"/>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
@@ -69346,6 +69450,7 @@
         <v>108.4</v>
       </c>
     </row>
+    <row r="78"/>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
@@ -69793,6 +69898,7 @@
         <v>187.1</v>
       </c>
     </row>
+    <row r="90"/>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
@@ -69976,6 +70082,7 @@
         <v>209.1</v>
       </c>
     </row>
+    <row r="96"/>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
@@ -70291,6 +70398,7 @@
         <v>223</v>
       </c>
     </row>
+    <row r="105"/>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
@@ -70353,6 +70461,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="108"/>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
@@ -70415,6 +70524,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="111"/>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
@@ -70554,6 +70664,7 @@
         <v>26</v>
       </c>
     </row>
+    <row r="116"/>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
@@ -70693,6 +70804,7 @@
         <v>27.6</v>
       </c>
     </row>
+    <row r="121"/>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
@@ -70900,6 +71012,7 @@
         <v>94</v>
       </c>
     </row>
+    <row r="129"/>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
@@ -71049,6 +71162,7 @@
         <v>74.40000000000001</v>
       </c>
     </row>
+    <row r="135"/>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
@@ -71546,6 +71660,7 @@
         <v>181.9</v>
       </c>
     </row>
+    <row r="153"/>
     <row r="154">
       <c r="A154" s="17" t="inlineStr">
         <is>
@@ -71714,6 +71829,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -71908,6 +72024,7 @@
         <v>63.8</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -72058,6 +72175,7 @@
         <v>153.6</v>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -72296,6 +72414,7 @@
         <v>93.2</v>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
@@ -72534,6 +72653,7 @@
         <v>72.8</v>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
@@ -72904,6 +73024,7 @@
         <v>196.5</v>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
@@ -73142,6 +73263,7 @@
         <v>172.4</v>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
@@ -73336,6 +73458,7 @@
         <v>172.4</v>
       </c>
     </row>
+    <row r="52"/>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
@@ -73574,6 +73697,7 @@
         <v>190.4</v>
       </c>
     </row>
+    <row r="59"/>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
@@ -73944,6 +74068,7 @@
         <v>192</v>
       </c>
     </row>
+    <row r="69"/>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
@@ -74182,6 +74307,7 @@
         <v>162.6</v>
       </c>
     </row>
+    <row r="76"/>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
@@ -74420,6 +74546,7 @@
         <v>68.3</v>
       </c>
     </row>
+    <row r="83"/>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
@@ -74746,6 +74873,7 @@
         <v>207.1</v>
       </c>
     </row>
+    <row r="92"/>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
@@ -74852,6 +74980,7 @@
         <v>19.6</v>
       </c>
     </row>
+    <row r="96"/>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
@@ -74972,6 +75101,7 @@
         <v>59.3</v>
       </c>
     </row>
+    <row r="101"/>
     <row r="102">
       <c r="A102" s="17" t="inlineStr">
         <is>
@@ -75272,6 +75402,7 @@
         <v>74.40000000000001</v>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -75466,6 +75597,7 @@
         <v>152.8</v>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -75640,6 +75772,7 @@
         <v>34.3</v>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -75911,6 +76044,7 @@
         <v>118.4</v>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
@@ -76105,6 +76239,7 @@
         <v>158.1</v>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
@@ -76167,6 +76302,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
@@ -76273,6 +76409,7 @@
         <v>14.3</v>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="17" t="inlineStr">
         <is>
@@ -76573,6 +76710,7 @@
         <v>64.2</v>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -76767,6 +76905,7 @@
         <v>69.09999999999999</v>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -76829,6 +76968,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -76891,6 +77031,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -77041,6 +77182,7 @@
         <v>34.3</v>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
@@ -77279,6 +77421,7 @@
         <v>73.59999999999999</v>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -77649,6 +77792,7 @@
         <v>154.9</v>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
@@ -77911,6 +78055,7 @@
         <v>88.7</v>
       </c>
     </row>
+    <row r="49"/>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
@@ -78457,6 +78602,7 @@
         <v>275.4</v>
       </c>
     </row>
+    <row r="63"/>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
@@ -78607,6 +78753,7 @@
         <v>59.3</v>
       </c>
     </row>
+    <row r="68"/>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
@@ -78937,6 +79084,7 @@
         <v>192</v>
       </c>
     </row>
+    <row r="78"/>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
@@ -79267,6 +79415,7 @@
         <v>221.9</v>
       </c>
     </row>
+    <row r="88"/>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
@@ -79637,6 +79786,7 @@
         <v>232.5</v>
       </c>
     </row>
+    <row r="98"/>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
@@ -80468,6 +80618,7 @@
         <v>448.1</v>
       </c>
     </row>
+    <row r="121"/>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
@@ -80569,6 +80720,7 @@
         <v>14.7</v>
       </c>
     </row>
+    <row r="125"/>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
@@ -80631,6 +80783,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="128"/>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
@@ -80693,6 +80846,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="131"/>
     <row r="132">
       <c r="A132" s="17" t="inlineStr">
         <is>
@@ -80856,6 +81010,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -80913,6 +81068,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -81151,6 +81307,7 @@
         <v>167.9</v>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -81345,6 +81502,7 @@
         <v>69.09999999999999</v>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
@@ -81539,6 +81697,7 @@
         <v>63.8</v>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
@@ -81733,6 +81892,7 @@
         <v>78.90000000000001</v>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
@@ -81883,6 +82043,7 @@
         <v>87.09999999999999</v>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
@@ -82154,6 +82315,7 @@
         <v>121.6</v>
       </c>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
@@ -82436,6 +82598,7 @@
         <v>125.5</v>
       </c>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
@@ -82674,6 +82837,7 @@
         <v>83.40000000000001</v>
       </c>
     </row>
+    <row r="60"/>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
@@ -83048,6 +83212,7 @@
         <v>240.2</v>
       </c>
     </row>
+    <row r="71"/>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
@@ -83198,6 +83363,7 @@
         <v>87.09999999999999</v>
       </c>
     </row>
+    <row r="76"/>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
@@ -83392,6 +83558,7 @@
         <v>91.59999999999999</v>
       </c>
     </row>
+    <row r="82"/>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
@@ -83542,6 +83709,7 @@
         <v>59.3</v>
       </c>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
@@ -83648,6 +83816,7 @@
         <v>19.6</v>
       </c>
     </row>
+    <row r="91"/>
     <row r="92">
       <c r="A92" s="17" t="inlineStr">
         <is>
@@ -83948,6 +84117,7 @@
         <v>183</v>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -84142,6 +84312,7 @@
         <v>74.40000000000001</v>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -84292,6 +84463,7 @@
         <v>64.59999999999999</v>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
@@ -84398,6 +84570,7 @@
         <v>54.8</v>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
@@ -84504,6 +84677,7 @@
         <v>18.8</v>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
@@ -84830,6 +85004,7 @@
         <v>135.3</v>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
@@ -84980,6 +85155,7 @@
         <v>81</v>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
@@ -85130,6 +85306,7 @@
         <v>59.3</v>
       </c>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
@@ -85357,6 +85534,7 @@
         <v>154.3</v>
       </c>
     </row>
+    <row r="52"/>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
@@ -85507,6 +85685,7 @@
         <v>81.8</v>
       </c>
     </row>
+    <row r="57"/>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
@@ -85701,6 +85880,7 @@
         <v>172.4</v>
       </c>
     </row>
+    <row r="63"/>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
@@ -85983,6 +86163,7 @@
         <v>88.7</v>
       </c>
     </row>
+    <row r="71"/>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
@@ -86210,6 +86391,7 @@
         <v>94.09999999999999</v>
       </c>
     </row>
+    <row r="78"/>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
@@ -86448,6 +86630,7 @@
         <v>68.7</v>
       </c>
     </row>
+    <row r="85"/>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
@@ -86719,6 +86902,7 @@
         <v>138.8</v>
       </c>
     </row>
+    <row r="93"/>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
@@ -86990,6 +87174,7 @@
         <v>131.1</v>
       </c>
     </row>
+    <row r="101"/>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
@@ -87305,6 +87490,7 @@
         <v>229.9</v>
       </c>
     </row>
+    <row r="110"/>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
@@ -87675,6 +87861,7 @@
         <v>196.5</v>
       </c>
     </row>
+    <row r="120"/>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
@@ -87957,6 +88144,7 @@
         <v>192</v>
       </c>
     </row>
+    <row r="128"/>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
@@ -88195,6 +88383,7 @@
         <v>172.4</v>
       </c>
     </row>
+    <row r="135"/>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
@@ -88433,6 +88622,7 @@
         <v>181.4</v>
       </c>
     </row>
+    <row r="142"/>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
@@ -88660,6 +88850,7 @@
         <v>121.3</v>
       </c>
     </row>
+    <row r="149"/>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
@@ -88854,6 +89045,7 @@
         <v>172.4</v>
       </c>
     </row>
+    <row r="155"/>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
@@ -88911,6 +89103,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="158"/>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
@@ -89105,6 +89298,7 @@
         <v>39.2</v>
       </c>
     </row>
+    <row r="164"/>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
@@ -89162,6 +89356,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="167"/>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
@@ -89268,6 +89463,7 @@
         <v>19.6</v>
       </c>
     </row>
+    <row r="171"/>
     <row r="172">
       <c r="A172" s="17" t="inlineStr">
         <is>
@@ -89524,6 +89720,7 @@
         <v>63</v>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -89620,6 +89817,7 @@
         <v>14.7</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -89716,6 +89914,7 @@
         <v>14.7</v>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -89778,6 +89977,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
@@ -89835,6 +90035,7 @@
         <v>9.800000000000001</v>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
@@ -90161,6 +90362,7 @@
         <v>92.40000000000001</v>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
@@ -90487,6 +90689,7 @@
         <v>53.1</v>
       </c>
     </row>
+    <row r="38"/>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
@@ -90637,6 +90840,7 @@
         <v>14.3</v>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
@@ -90875,6 +91079,7 @@
         <v>84.2</v>
       </c>
     </row>
+    <row r="50"/>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
@@ -91069,6 +91274,7 @@
         <v>64.2</v>
       </c>
     </row>
+    <row r="56"/>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
@@ -91219,6 +91425,7 @@
         <v>69.09999999999999</v>
       </c>
     </row>
+    <row r="61"/>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
@@ -91457,6 +91664,7 @@
         <v>82.59999999999999</v>
       </c>
     </row>
+    <row r="68"/>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
@@ -91651,6 +91859,7 @@
         <v>74.40000000000001</v>
       </c>
     </row>
+    <row r="74"/>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
@@ -91878,6 +92087,7 @@
         <v>87.8</v>
       </c>
     </row>
+    <row r="81"/>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
@@ -92336,6 +92546,7 @@
         <v>241</v>
       </c>
     </row>
+    <row r="93"/>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
@@ -92574,6 +92785,7 @@
         <v>73.59999999999999</v>
       </c>
     </row>
+    <row r="100"/>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
@@ -92768,6 +92980,7 @@
         <v>104.3</v>
       </c>
     </row>
+    <row r="106"/>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
@@ -92995,6 +93208,7 @@
         <v>87.8</v>
       </c>
     </row>
+    <row r="113"/>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
@@ -93189,6 +93403,7 @@
         <v>104.3</v>
       </c>
     </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
@@ -93329,6 +93544,7 @@
         <v>24.1</v>
       </c>
     </row>
+    <row r="124"/>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
@@ -93420,6 +93636,7 @@
         <v>54.8</v>
       </c>
     </row>
+    <row r="128"/>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
@@ -93540,6 +93757,7 @@
         <v>64.59999999999999</v>
       </c>
     </row>
+    <row r="133"/>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
@@ -93660,6 +93878,7 @@
         <v>59.3</v>
       </c>
     </row>
+    <row r="138"/>
     <row r="139">
       <c r="A139" s="17" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Separate SUSHICORP into its own database, distinct from KFC group
SUSHICORP (KOBE/NOE, RUC 1792256267001) is a separate company from the
KFC group and now lives in its own BASE_DATOS_SUSHICORP.xlsx (13 locals,
62 extinguishers). Removed all 13 KN locals from BASE_DATOS_KFC.xlsx,
which now holds only the KFC group (197 locals). Verified zero crossover:
no KN in KFC, no KFC marca in SUSHICORP, totals match each summary exactly.

The app now loads both bases and merges them in the monthly plan (each
local keeps its own company/RUC for invoicing). Also handles the grouped
DETALLE format via forward-fill (recovers extinguishers that were
previously dropped) and separates MOVILIZACIÓN rows as viáticos.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFXpAjF8wqo1CCwLa1Q85Z
</commit_message>
<xml_diff>
--- a/BASE_DATOS_KFC.xlsx
+++ b/BASE_DATOS_KFC.xlsx
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J211"/>
+  <dimension ref="A1:J198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8520,526 +8520,6 @@
         <v>2023</v>
       </c>
       <c r="J198" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>KN001</t>
-        </is>
-      </c>
-      <c r="B199" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C199" t="inlineStr">
-        <is>
-          <t>KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="D199" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="E199" t="n">
-        <v>6</v>
-      </c>
-      <c r="F199" t="n">
-        <v>40</v>
-      </c>
-      <c r="G199" t="n">
-        <v>94</v>
-      </c>
-      <c r="H199" t="n">
-        <v>94</v>
-      </c>
-      <c r="I199" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J199" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>KN002</t>
-        </is>
-      </c>
-      <c r="B200" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C200" t="inlineStr">
-        <is>
-          <t>KN02 - NOE BOCCA SAMBO</t>
-        </is>
-      </c>
-      <c r="D200" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="E200" t="n">
-        <v>4</v>
-      </c>
-      <c r="F200" t="n">
-        <v>32</v>
-      </c>
-      <c r="G200" t="n">
-        <v>74.40000000000001</v>
-      </c>
-      <c r="H200" t="n">
-        <v>74.40000000000001</v>
-      </c>
-      <c r="I200" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J200" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>KN003</t>
-        </is>
-      </c>
-      <c r="B201" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C201" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="D201" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="E201" t="n">
-        <v>16</v>
-      </c>
-      <c r="F201" t="n">
-        <v>78</v>
-      </c>
-      <c r="G201" t="n">
-        <v>181.9</v>
-      </c>
-      <c r="H201" t="n">
-        <v>181.9</v>
-      </c>
-      <c r="I201" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J201" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>KN004</t>
-        </is>
-      </c>
-      <c r="B202" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C202" t="inlineStr">
-        <is>
-          <t>KN04 - KOBE SUPERCINES ORELLANA</t>
-        </is>
-      </c>
-      <c r="D202" t="inlineStr">
-        <is>
-          <t>MARZO</t>
-        </is>
-      </c>
-      <c r="E202" t="n">
-        <v>3</v>
-      </c>
-      <c r="F202" t="n">
-        <v>26</v>
-      </c>
-      <c r="G202" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="H202" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="I202" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J202" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>KN005</t>
-        </is>
-      </c>
-      <c r="B203" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C203" t="inlineStr">
-        <is>
-          <t>KN05 - KOBE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="D203" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="E203" t="n">
-        <v>2</v>
-      </c>
-      <c r="F203" t="n">
-        <v>24</v>
-      </c>
-      <c r="G203" t="n">
-        <v>54.8</v>
-      </c>
-      <c r="H203" t="n">
-        <v>54.8</v>
-      </c>
-      <c r="I203" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J203" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="inlineStr">
-        <is>
-          <t>KN006</t>
-        </is>
-      </c>
-      <c r="B204" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C204" t="inlineStr">
-        <is>
-          <t>KN06 - KOBE PLAZA BATAN</t>
-        </is>
-      </c>
-      <c r="D204" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="E204" t="n">
-        <v>3</v>
-      </c>
-      <c r="F204" t="n">
-        <v>28</v>
-      </c>
-      <c r="G204" t="n">
-        <v>64.59999999999999</v>
-      </c>
-      <c r="H204" t="n">
-        <v>64.59999999999999</v>
-      </c>
-      <c r="I204" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J204" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="inlineStr">
-        <is>
-          <t>KN007</t>
-        </is>
-      </c>
-      <c r="B205" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C205" t="inlineStr">
-        <is>
-          <t>KN07 - KOBE MALL DEL NORTE</t>
-        </is>
-      </c>
-      <c r="D205" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="E205" t="n">
-        <v>3</v>
-      </c>
-      <c r="F205" t="n">
-        <v>26</v>
-      </c>
-      <c r="G205" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="H205" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="I205" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J205" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>KN008</t>
-        </is>
-      </c>
-      <c r="B206" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C206" t="inlineStr">
-        <is>
-          <t>KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="D206" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="E206" t="n">
-        <v>5</v>
-      </c>
-      <c r="F206" t="n">
-        <v>42</v>
-      </c>
-      <c r="G206" t="n">
-        <v>81.09999999999999</v>
-      </c>
-      <c r="H206" t="n">
-        <v>81.09999999999999</v>
-      </c>
-      <c r="I206" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J206" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>KN009</t>
-        </is>
-      </c>
-      <c r="B207" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C207" t="inlineStr">
-        <is>
-          <t>KN09 - KOBE PLAZA TIA JOYA</t>
-        </is>
-      </c>
-      <c r="D207" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="E207" t="n">
-        <v>3</v>
-      </c>
-      <c r="F207" t="n">
-        <v>26</v>
-      </c>
-      <c r="G207" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="H207" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="I207" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J207" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>KN010</t>
-        </is>
-      </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C208" t="inlineStr">
-        <is>
-          <t>KN10 - KOBE BAMBOO PLAZA VIA A LA C</t>
-        </is>
-      </c>
-      <c r="D208" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="E208" t="n">
-        <v>3</v>
-      </c>
-      <c r="F208" t="n">
-        <v>24</v>
-      </c>
-      <c r="G208" t="n">
-        <v>54</v>
-      </c>
-      <c r="H208" t="n">
-        <v>54</v>
-      </c>
-      <c r="I208" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J208" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>KN011</t>
-        </is>
-      </c>
-      <c r="B209" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C209" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="D209" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="E209" t="n">
-        <v>8</v>
-      </c>
-      <c r="F209" t="n">
-        <v>56</v>
-      </c>
-      <c r="G209" t="n">
-        <v>133.2</v>
-      </c>
-      <c r="H209" t="n">
-        <v>133.2</v>
-      </c>
-      <c r="I209" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J209" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="inlineStr">
-        <is>
-          <t>KN012</t>
-        </is>
-      </c>
-      <c r="B210" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C210" t="inlineStr">
-        <is>
-          <t>KN12 - KOBE RIOC ENTRE RIOS</t>
-        </is>
-      </c>
-      <c r="D210" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="E210" t="n">
-        <v>3</v>
-      </c>
-      <c r="F210" t="n">
-        <v>26</v>
-      </c>
-      <c r="G210" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="H210" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="I210" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J210" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>KN013</t>
-        </is>
-      </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C211" t="inlineStr">
-        <is>
-          <t>KN13 - KOBE RIOC CEIBOS</t>
-        </is>
-      </c>
-      <c r="D211" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="E211" t="n">
-        <v>3</v>
-      </c>
-      <c r="F211" t="n">
-        <v>26</v>
-      </c>
-      <c r="G211" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="H211" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="I211" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J211" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -26670,7 +26150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1450"/>
+  <dimension ref="A1:J1326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -69835,4188 +69315,18 @@
         <v>9.800000000000001</v>
       </c>
     </row>
-    <row r="1315">
-      <c r="D1315" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1315" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1315" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1315" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1315" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1315" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1315" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1316">
-      <c r="E1316" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1316" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1316" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1316" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1316" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1316" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1317">
-      <c r="D1317" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1317" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1317" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1317" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1317" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1317" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1317" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1318">
-      <c r="D1318" t="inlineStr">
-        <is>
-          <t>GABINETE ENTRADA</t>
-        </is>
-      </c>
-      <c r="E1318" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1318" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1318" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1318" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1318" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1318" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1319">
-      <c r="D1319" t="inlineStr">
-        <is>
-          <t>BODEGA</t>
-        </is>
-      </c>
-      <c r="E1319" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1319" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1319" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1319" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1319" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1319" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1320">
-      <c r="A1320" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="F1320" t="inlineStr">
-        <is>
-          <t>6 ext.</t>
-        </is>
-      </c>
-      <c r="G1320" t="n">
-        <v>40</v>
-      </c>
-      <c r="H1320" t="n">
-        <v>94</v>
-      </c>
-    </row>
+    <row r="1315"/>
+    <row r="1316"/>
+    <row r="1317"/>
+    <row r="1318"/>
+    <row r="1319"/>
+    <row r="1320"/>
     <row r="1321"/>
-    <row r="1322">
-      <c r="D1322" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1322" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1322" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1322" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1322" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1322" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1322" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1323">
-      <c r="D1323" t="inlineStr">
-        <is>
-          <t>BODEGA</t>
-        </is>
-      </c>
-      <c r="E1323" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1323" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1323" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1323" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1323" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1323" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1324">
-      <c r="D1324" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1324" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1324" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1324" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1324" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1324" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1324" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1325">
-      <c r="A1325" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN02 - NOE BOCCA SAMBO</t>
-        </is>
-      </c>
-      <c r="F1325" t="inlineStr">
-        <is>
-          <t>4 ext.</t>
-        </is>
-      </c>
-      <c r="G1325" t="n">
-        <v>32</v>
-      </c>
-      <c r="H1325" t="n">
-        <v>74.40000000000001</v>
-      </c>
-    </row>
+    <row r="1322"/>
+    <row r="1323"/>
+    <row r="1324"/>
+    <row r="1325"/>
     <row r="1326"/>
-    <row r="1327">
-      <c r="D1327" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1327" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1327" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1327" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1327" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1327" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1327" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1328">
-      <c r="D1328" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1328" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1328" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1328" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1328" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1328" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1328" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1329">
-      <c r="D1329" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1329" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1329" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1329" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1329" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1329" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1329" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1330">
-      <c r="D1330" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1330" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1330" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1330" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1330" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1330" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1330" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1331">
-      <c r="D1331" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1331" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1331" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1331" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1331" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1331" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1331" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1332">
-      <c r="D1332" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1332" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1332" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1332" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1332" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1332" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1332" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1333">
-      <c r="D1333" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1333" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1333" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1333" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1333" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1333" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1333" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1334">
-      <c r="D1334" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1334" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1334" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1334" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1334" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1334" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1334" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1335">
-      <c r="D1335" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1335" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1335" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1335" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1335" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1335" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1335" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1336">
-      <c r="D1336" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1336" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1336" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1336" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1336" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="I1336" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1336" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1337">
-      <c r="D1337" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1337" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1337" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1337" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1337" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="I1337" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1337" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1338">
-      <c r="D1338" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1338" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1338" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1338" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1338" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1338" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1338" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1339">
-      <c r="D1339" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1339" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1339" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1339" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1339" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1339" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1339" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1340">
-      <c r="D1340" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1340" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1340" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1340" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1340" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1340" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1340" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1341">
-      <c r="D1341" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1341" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1341" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1341" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1341" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1341" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1341" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1342">
-      <c r="A1342" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="F1342" t="inlineStr">
-        <is>
-          <t>16 ext.</t>
-        </is>
-      </c>
-      <c r="G1342" t="n">
-        <v>78</v>
-      </c>
-      <c r="H1342" t="n">
-        <v>181.9</v>
-      </c>
-    </row>
-    <row r="1343"/>
-    <row r="1344">
-      <c r="D1344" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1344" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1344" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1344" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1344" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1344" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1344" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1345">
-      <c r="D1345" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1345" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1345" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1345" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1345" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1345" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1345" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1346">
-      <c r="A1346" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN04 - KOBE SUPERCINES ORELLANA</t>
-        </is>
-      </c>
-      <c r="F1346" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1346" t="n">
-        <v>26</v>
-      </c>
-      <c r="H1346" t="n">
-        <v>59.3</v>
-      </c>
-    </row>
-    <row r="1347"/>
-    <row r="1348">
-      <c r="D1348" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1348" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1348" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1348" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1348" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1348" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1348" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1349">
-      <c r="A1349" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN05 - KOBE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="F1349" t="inlineStr">
-        <is>
-          <t>2 ext.</t>
-        </is>
-      </c>
-      <c r="G1349" t="n">
-        <v>24</v>
-      </c>
-      <c r="H1349" t="n">
-        <v>54.8</v>
-      </c>
-    </row>
-    <row r="1350"/>
-    <row r="1351">
-      <c r="D1351" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1351" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1351" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1351" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1351" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1351" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1351" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1352">
-      <c r="D1352" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1352" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1352" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1352" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1352" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1352" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1352" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1353">
-      <c r="A1353" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN06 - KOBE PLAZA BATAN</t>
-        </is>
-      </c>
-      <c r="F1353" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1353" t="n">
-        <v>28</v>
-      </c>
-      <c r="H1353" t="n">
-        <v>64.59999999999999</v>
-      </c>
-    </row>
-    <row r="1354"/>
-    <row r="1355">
-      <c r="D1355" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1355" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1355" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1355" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1355" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1355" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1355" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1356">
-      <c r="D1356" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1356" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1356" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1356" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1356" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1356" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1356" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1357">
-      <c r="A1357" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN07 - KOBE MALL DEL NORTE</t>
-        </is>
-      </c>
-      <c r="F1357" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1357" t="n">
-        <v>26</v>
-      </c>
-      <c r="H1357" t="n">
-        <v>59.3</v>
-      </c>
-    </row>
-    <row r="1358"/>
-    <row r="1359">
-      <c r="D1359" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1359" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1359" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1359" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1359" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1359" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1359" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1360">
-      <c r="D1360" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1360" t="inlineStr">
-        <is>
-          <t>TIPO K</t>
-        </is>
-      </c>
-      <c r="F1360" t="inlineStr">
-        <is>
-          <t>2.5 GLS</t>
-        </is>
-      </c>
-      <c r="G1360" t="n">
-        <v>12</v>
-      </c>
-      <c r="H1360" t="n">
-        <v>12</v>
-      </c>
-      <c r="I1360" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1360" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1361">
-      <c r="D1361" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1361" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1361" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1361" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1361" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1361" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1361" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1362">
-      <c r="D1362" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1362" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1362" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1362" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1362" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1362" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1362" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1363">
-      <c r="A1363" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="F1363" t="inlineStr">
-        <is>
-          <t>5 ext.</t>
-        </is>
-      </c>
-      <c r="G1363" t="n">
-        <v>42</v>
-      </c>
-      <c r="H1363" t="n">
-        <v>81.09999999999999</v>
-      </c>
-    </row>
-    <row r="1364"/>
-    <row r="1365">
-      <c r="D1365" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1365" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1365" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1365" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1365" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1365" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1365" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1366">
-      <c r="D1366" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1366" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1366" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1366" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1366" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1366" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1366" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1367">
-      <c r="A1367" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN09 - KOBE PLAZA TIA JOYA</t>
-        </is>
-      </c>
-      <c r="F1367" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1367" t="n">
-        <v>26</v>
-      </c>
-      <c r="H1367" t="n">
-        <v>59.3</v>
-      </c>
-    </row>
-    <row r="1368"/>
-    <row r="1369">
-      <c r="D1369" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1369" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1369" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1369" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1369" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1369" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1369" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1370">
-      <c r="D1370" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1370" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1370" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1370" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1370" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1370" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1370" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1371">
-      <c r="A1371" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN10 - KOBE BAMBOO PLAZA VIA A LA C</t>
-        </is>
-      </c>
-      <c r="F1371" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1371" t="n">
-        <v>24</v>
-      </c>
-      <c r="H1371" t="n">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="1372"/>
-    <row r="1373">
-      <c r="D1373" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1373" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1373" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1373" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1373" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="I1373" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1373" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1374">
-      <c r="D1374" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1374" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1374" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1374" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1374" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="I1374" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1374" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1375">
-      <c r="D1375" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1375" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1375" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1375" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1375" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1375" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1375" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1376">
-      <c r="D1376" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1376" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1376" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1376" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1376" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1376" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1376" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1377">
-      <c r="D1377" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1377" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1377" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1377" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1377" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1377" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1377" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1378">
-      <c r="D1378" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1378" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1378" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1378" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1378" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1378" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1378" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1379">
-      <c r="D1379" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1379" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1379" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1379" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1379" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1379" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1379" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1380">
-      <c r="A1380" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="F1380" t="inlineStr">
-        <is>
-          <t>8 ext.</t>
-        </is>
-      </c>
-      <c r="G1380" t="n">
-        <v>56</v>
-      </c>
-      <c r="H1380" t="n">
-        <v>133.2</v>
-      </c>
-    </row>
-    <row r="1381"/>
-    <row r="1382">
-      <c r="D1382" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1382" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1382" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1382" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1382" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1382" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1382" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1383">
-      <c r="D1383" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1383" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1383" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1383" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1383" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1383" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1383" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1384">
-      <c r="A1384" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN12 - KOBE RIOC ENTRE RIOS</t>
-        </is>
-      </c>
-      <c r="F1384" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1384" t="n">
-        <v>26</v>
-      </c>
-      <c r="H1384" t="n">
-        <v>59.3</v>
-      </c>
-    </row>
-    <row r="1385"/>
-    <row r="1386">
-      <c r="D1386" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1386" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1386" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1386" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1386" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1386" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1386" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1387">
-      <c r="D1387" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1387" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1387" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1387" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1387" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1387" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1387" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1388">
-      <c r="A1388" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN13 - KOBE RIOC CEIBOS</t>
-        </is>
-      </c>
-      <c r="F1388" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1388" t="n">
-        <v>26</v>
-      </c>
-      <c r="H1388" t="n">
-        <v>59.3</v>
-      </c>
-    </row>
-    <row r="1389">
-      <c r="A1389" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1389" t="inlineStr">
-        <is>
-          <t>KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1389" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1389" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1389" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1389" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1389" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1389" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1389" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1389" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1390">
-      <c r="A1390" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1390" t="inlineStr">
-        <is>
-          <t>KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1390" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1390" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1390" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1390" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1390" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1390" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1390" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1390" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1391">
-      <c r="A1391" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1391" t="inlineStr">
-        <is>
-          <t>KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1391" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1391" t="inlineStr">
-        <is>
-          <t>OFICINA</t>
-        </is>
-      </c>
-      <c r="E1391" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1391" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1391" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1391" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1391" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1391" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1392">
-      <c r="A1392" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1392" t="inlineStr">
-        <is>
-          <t>KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1392" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1392" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1392" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1392" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1392" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1392" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1392" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1392" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1393">
-      <c r="A1393" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1393" t="inlineStr">
-        <is>
-          <t>KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1393" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1393" t="inlineStr">
-        <is>
-          <t>GABINETE ENTRADA PRINCIPAÑ</t>
-        </is>
-      </c>
-      <c r="E1393" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1393" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1393" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1393" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1393" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1393" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1394">
-      <c r="A1394" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1394" t="inlineStr">
-        <is>
-          <t>KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1394" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1394" t="inlineStr">
-        <is>
-          <t>BODEGA P/B</t>
-        </is>
-      </c>
-      <c r="E1394" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1394" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1394" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1394" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1394" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1394" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1395">
-      <c r="A1395" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1395" t="inlineStr">
-        <is>
-          <t>KN02 - NOE BOCCA SAMBO</t>
-        </is>
-      </c>
-      <c r="C1395" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1395" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1395" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1395" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1395" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1395" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1395" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1395" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1396">
-      <c r="A1396" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1396" t="inlineStr">
-        <is>
-          <t>KN02 - NOE BOCCA SAMBO</t>
-        </is>
-      </c>
-      <c r="C1396" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1396" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1396" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1396" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1396" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1396" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1396" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1396" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1397">
-      <c r="A1397" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1397" t="inlineStr">
-        <is>
-          <t>KN02 - NOE BOCCA SAMBO</t>
-        </is>
-      </c>
-      <c r="C1397" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1397" t="inlineStr">
-        <is>
-          <t>BODEGA</t>
-        </is>
-      </c>
-      <c r="E1397" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1397" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1397" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1397" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1397" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1397" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1398">
-      <c r="A1398" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1398" t="inlineStr">
-        <is>
-          <t>KN02 - NOE BOCCA SAMBO</t>
-        </is>
-      </c>
-      <c r="C1398" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1398" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1398" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1398" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1398" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1398" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1398" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1398" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1399">
-      <c r="A1399" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1399" t="inlineStr">
-        <is>
-          <t>KN04 - KOBE SUPERCINES ORELLANA</t>
-        </is>
-      </c>
-      <c r="C1399" t="inlineStr">
-        <is>
-          <t>MARZO</t>
-        </is>
-      </c>
-      <c r="D1399" t="inlineStr"/>
-      <c r="E1399" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1399" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1399" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1399" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1399" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1399" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1400">
-      <c r="A1400" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1400" t="inlineStr">
-        <is>
-          <t>KN04 - KOBE SUPERCINES ORELLANA</t>
-        </is>
-      </c>
-      <c r="C1400" t="inlineStr">
-        <is>
-          <t>MARZO</t>
-        </is>
-      </c>
-      <c r="D1400" t="inlineStr"/>
-      <c r="E1400" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1400" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1400" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1400" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1400" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1400" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1401">
-      <c r="A1401" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1401" t="inlineStr">
-        <is>
-          <t>KN04 - KOBE SUPERCINES ORELLANA</t>
-        </is>
-      </c>
-      <c r="C1401" t="inlineStr">
-        <is>
-          <t>MARZO</t>
-        </is>
-      </c>
-      <c r="D1401" t="inlineStr"/>
-      <c r="E1401" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1401" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1401" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1401" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1401" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1401" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1402">
-      <c r="A1402" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1402" t="inlineStr">
-        <is>
-          <t>KN06 - KOBE PLAZA BATAN</t>
-        </is>
-      </c>
-      <c r="C1402" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1402" t="inlineStr"/>
-      <c r="E1402" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1402" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1402" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1402" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1402" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1402" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1403">
-      <c r="A1403" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1403" t="inlineStr">
-        <is>
-          <t>KN06 - KOBE PLAZA BATAN</t>
-        </is>
-      </c>
-      <c r="C1403" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1403" t="inlineStr"/>
-      <c r="E1403" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1403" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1403" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1403" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1403" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1403" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1404">
-      <c r="A1404" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1404" t="inlineStr">
-        <is>
-          <t>KN06 - KOBE PLAZA BATAN</t>
-        </is>
-      </c>
-      <c r="C1404" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1404" t="inlineStr"/>
-      <c r="E1404" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1404" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1404" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1404" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1404" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1404" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1405">
-      <c r="A1405" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1405" t="inlineStr">
-        <is>
-          <t>KN05 - KOBE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1405" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1405" t="inlineStr"/>
-      <c r="E1405" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1405" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1405" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1405" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1405" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1405" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1406">
-      <c r="A1406" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1406" t="inlineStr">
-        <is>
-          <t>KN05 - KOBE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1406" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1406" t="inlineStr"/>
-      <c r="E1406" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1406" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1406" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1406" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1406" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1406" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1407">
-      <c r="A1407" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1407" t="inlineStr">
-        <is>
-          <t>KN07 - KOBE MALL DEL NORTE</t>
-        </is>
-      </c>
-      <c r="C1407" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1407" t="inlineStr"/>
-      <c r="E1407" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1407" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1407" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1407" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1407" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1407" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1408">
-      <c r="A1408" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1408" t="inlineStr">
-        <is>
-          <t>KN07 - KOBE MALL DEL NORTE</t>
-        </is>
-      </c>
-      <c r="C1408" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1408" t="inlineStr"/>
-      <c r="E1408" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1408" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1408" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1408" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1408" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1408" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1409">
-      <c r="A1409" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1409" t="inlineStr">
-        <is>
-          <t>KN07 - KOBE MALL DEL NORTE</t>
-        </is>
-      </c>
-      <c r="C1409" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1409" t="inlineStr"/>
-      <c r="E1409" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1409" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1409" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1409" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1409" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1409" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1410">
-      <c r="A1410" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1410" t="inlineStr">
-        <is>
-          <t>KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="C1410" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1410" t="inlineStr"/>
-      <c r="E1410" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1410" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1410" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1410" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1410" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1410" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1411">
-      <c r="A1411" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1411" t="inlineStr">
-        <is>
-          <t>KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="C1411" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1411" t="inlineStr"/>
-      <c r="E1411" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1411" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1411" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1411" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1411" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1411" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1412">
-      <c r="A1412" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1412" t="inlineStr">
-        <is>
-          <t>KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="C1412" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1412" t="inlineStr"/>
-      <c r="E1412" t="inlineStr">
-        <is>
-          <t>TIPO K</t>
-        </is>
-      </c>
-      <c r="F1412" t="inlineStr">
-        <is>
-          <t>2.5 GLS</t>
-        </is>
-      </c>
-      <c r="G1412" t="n">
-        <v>12</v>
-      </c>
-      <c r="H1412" t="n">
-        <v>12</v>
-      </c>
-      <c r="I1412" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1412" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1413">
-      <c r="A1413" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1413" t="inlineStr">
-        <is>
-          <t>KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="C1413" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1413" t="inlineStr"/>
-      <c r="E1413" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1413" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1413" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1413" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1413" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1413" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1414">
-      <c r="A1414" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1414" t="inlineStr">
-        <is>
-          <t>KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="C1414" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1414" t="inlineStr"/>
-      <c r="E1414" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1414" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1414" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1414" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1414" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1414" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1415">
-      <c r="A1415" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1415" t="inlineStr">
-        <is>
-          <t>KN09 - KOBE PLAZA TIA JOYA</t>
-        </is>
-      </c>
-      <c r="C1415" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1415" t="inlineStr"/>
-      <c r="E1415" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1415" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1415" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1415" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1415" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1415" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1416">
-      <c r="A1416" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1416" t="inlineStr">
-        <is>
-          <t>KN09 - KOBE PLAZA TIA JOYA</t>
-        </is>
-      </c>
-      <c r="C1416" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1416" t="inlineStr"/>
-      <c r="E1416" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1416" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1416" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1416" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1416" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1416" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1417">
-      <c r="A1417" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1417" t="inlineStr">
-        <is>
-          <t>KN09 - KOBE PLAZA TIA JOYA</t>
-        </is>
-      </c>
-      <c r="C1417" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1417" t="inlineStr"/>
-      <c r="E1417" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1417" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1417" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1417" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1417" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1417" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1418">
-      <c r="A1418" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1418" t="inlineStr">
-        <is>
-          <t>KN10 - KOBE BAMBOO PLAZA VIA A LA C</t>
-        </is>
-      </c>
-      <c r="C1418" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1418" t="inlineStr"/>
-      <c r="E1418" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1418" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1418" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1418" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1418" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1418" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1419">
-      <c r="A1419" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1419" t="inlineStr">
-        <is>
-          <t>KN10 - KOBE BAMBOO PLAZA VIA A LA C</t>
-        </is>
-      </c>
-      <c r="C1419" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1419" t="inlineStr"/>
-      <c r="E1419" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1419" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1419" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1419" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1419" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1419" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1420">
-      <c r="A1420" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1420" t="inlineStr">
-        <is>
-          <t>KN10 - KOBE BAMBOO PLAZA VIA A LA C</t>
-        </is>
-      </c>
-      <c r="C1420" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1420" t="inlineStr"/>
-      <c r="E1420" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1420" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1420" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1420" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1420" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1420" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1421">
-      <c r="A1421" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1421" t="inlineStr">
-        <is>
-          <t>KN12 - KOBE RIOC ENTRE RIOS</t>
-        </is>
-      </c>
-      <c r="C1421" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1421" t="inlineStr"/>
-      <c r="E1421" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1421" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1421" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1421" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1421" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1421" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1422">
-      <c r="A1422" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1422" t="inlineStr">
-        <is>
-          <t>KN12 - KOBE RIOC ENTRE RIOS</t>
-        </is>
-      </c>
-      <c r="C1422" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1422" t="inlineStr"/>
-      <c r="E1422" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1422" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1422" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1422" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1422" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1422" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1423">
-      <c r="A1423" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1423" t="inlineStr">
-        <is>
-          <t>KN12 - KOBE RIOC ENTRE RIOS</t>
-        </is>
-      </c>
-      <c r="C1423" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1423" t="inlineStr"/>
-      <c r="E1423" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1423" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1423" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1423" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1423" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1423" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1424">
-      <c r="A1424" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1424" t="inlineStr">
-        <is>
-          <t>KN13 - KOBE RIOC CEIBOS</t>
-        </is>
-      </c>
-      <c r="C1424" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1424" t="inlineStr"/>
-      <c r="E1424" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1424" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1424" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1424" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1424" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1424" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1425">
-      <c r="A1425" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1425" t="inlineStr">
-        <is>
-          <t>KN13 - KOBE RIOC CEIBOS</t>
-        </is>
-      </c>
-      <c r="C1425" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1425" t="inlineStr"/>
-      <c r="E1425" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1425" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1425" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1425" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1425" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1425" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1426">
-      <c r="A1426" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1426" t="inlineStr">
-        <is>
-          <t>KN13 - KOBE RIOC CEIBOS</t>
-        </is>
-      </c>
-      <c r="C1426" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1426" t="inlineStr"/>
-      <c r="E1426" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1426" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1426" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1426" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1426" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1426" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1427">
-      <c r="A1427" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1427" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1427" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1427" t="inlineStr"/>
-      <c r="E1427" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1427" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1427" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1427" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1427" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1427" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1428">
-      <c r="A1428" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1428" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1428" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1428" t="inlineStr"/>
-      <c r="E1428" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1428" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1428" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1428" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="I1428" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1428" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1429">
-      <c r="A1429" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1429" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1429" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1429" t="inlineStr"/>
-      <c r="E1429" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1429" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1429" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1429" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="I1429" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1429" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1430">
-      <c r="A1430" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1430" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1430" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1430" t="inlineStr"/>
-      <c r="E1430" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1430" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1430" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1430" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1430" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1430" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1431">
-      <c r="A1431" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1431" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1431" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1431" t="inlineStr"/>
-      <c r="E1431" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1431" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1431" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1431" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1431" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1431" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1432">
-      <c r="A1432" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1432" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1432" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1432" t="inlineStr"/>
-      <c r="E1432" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1432" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1432" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1432" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1432" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1432" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1433">
-      <c r="A1433" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1433" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1433" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1433" t="inlineStr"/>
-      <c r="E1433" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1433" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1433" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1433" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1433" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1433" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1434">
-      <c r="A1434" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1434" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1434" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1434" t="inlineStr"/>
-      <c r="E1434" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1434" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1434" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1434" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1434" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1434" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1435">
-      <c r="A1435" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1435" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1435" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1435" t="inlineStr"/>
-      <c r="E1435" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1435" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1435" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1435" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1435" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1435" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1436">
-      <c r="A1436" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1436" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1436" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1436" t="inlineStr"/>
-      <c r="E1436" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1436" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1436" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1436" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1436" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1436" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1437">
-      <c r="A1437" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1437" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1437" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1437" t="inlineStr"/>
-      <c r="E1437" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1437" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1437" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1437" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1437" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1437" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1438">
-      <c r="A1438" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1438" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1438" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1438" t="inlineStr"/>
-      <c r="E1438" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1438" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1438" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1438" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1438" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1438" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1439">
-      <c r="A1439" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1439" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1439" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1439" t="inlineStr"/>
-      <c r="E1439" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1439" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1439" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1439" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1439" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1439" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1440">
-      <c r="A1440" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1440" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1440" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1440" t="inlineStr"/>
-      <c r="E1440" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1440" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1440" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1440" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1440" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1440" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1441">
-      <c r="A1441" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1441" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1441" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1441" t="inlineStr"/>
-      <c r="E1441" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1441" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1441" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1441" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1441" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1441" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1442">
-      <c r="A1442" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1442" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1442" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1442" t="inlineStr"/>
-      <c r="E1442" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1442" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1442" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1442" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1442" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1442" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1443">
-      <c r="A1443" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1443" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1443" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1443" t="inlineStr"/>
-      <c r="E1443" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1443" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1443" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1443" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1443" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1443" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1444">
-      <c r="A1444" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1444" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1444" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1444" t="inlineStr"/>
-      <c r="E1444" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1444" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1444" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1444" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1444" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1444" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1445">
-      <c r="A1445" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1445" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1445" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1445" t="inlineStr"/>
-      <c r="E1445" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1445" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1445" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1445" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="I1445" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1445" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1446">
-      <c r="A1446" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1446" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1446" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1446" t="inlineStr"/>
-      <c r="E1446" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1446" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1446" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1446" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="I1446" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1446" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1447">
-      <c r="A1447" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1447" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1447" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1447" t="inlineStr"/>
-      <c r="E1447" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1447" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1447" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1447" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1447" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1447" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1448">
-      <c r="A1448" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1448" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1448" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1448" t="inlineStr"/>
-      <c r="E1448" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1448" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1448" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1448" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1448" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1448" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1449">
-      <c r="A1449" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1449" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1449" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1449" t="inlineStr"/>
-      <c r="E1449" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1449" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1449" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1449" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1449" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1449" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1450">
-      <c r="A1450" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1450" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1450" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1450" t="inlineStr"/>
-      <c r="E1450" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1450" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1450" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1450" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1450" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1450" t="n">
-        <v>2026</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ alejosl0801/previfuego-facturacion@5e4456d9cd46c738d7345f2f68662c1c3d2f72da 🚀
</commit_message>
<xml_diff>
--- a/BASE_DATOS_KFC.xlsx
+++ b/BASE_DATOS_KFC.xlsx
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J211"/>
+  <dimension ref="A1:J198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8520,526 +8520,6 @@
         <v>2023</v>
       </c>
       <c r="J198" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>KN001</t>
-        </is>
-      </c>
-      <c r="B199" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C199" t="inlineStr">
-        <is>
-          <t>KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="D199" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="E199" t="n">
-        <v>6</v>
-      </c>
-      <c r="F199" t="n">
-        <v>40</v>
-      </c>
-      <c r="G199" t="n">
-        <v>94</v>
-      </c>
-      <c r="H199" t="n">
-        <v>94</v>
-      </c>
-      <c r="I199" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J199" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>KN002</t>
-        </is>
-      </c>
-      <c r="B200" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C200" t="inlineStr">
-        <is>
-          <t>KN02 - NOE BOCCA SAMBO</t>
-        </is>
-      </c>
-      <c r="D200" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="E200" t="n">
-        <v>4</v>
-      </c>
-      <c r="F200" t="n">
-        <v>32</v>
-      </c>
-      <c r="G200" t="n">
-        <v>74.40000000000001</v>
-      </c>
-      <c r="H200" t="n">
-        <v>74.40000000000001</v>
-      </c>
-      <c r="I200" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J200" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>KN003</t>
-        </is>
-      </c>
-      <c r="B201" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C201" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="D201" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="E201" t="n">
-        <v>16</v>
-      </c>
-      <c r="F201" t="n">
-        <v>78</v>
-      </c>
-      <c r="G201" t="n">
-        <v>181.9</v>
-      </c>
-      <c r="H201" t="n">
-        <v>181.9</v>
-      </c>
-      <c r="I201" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J201" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>KN004</t>
-        </is>
-      </c>
-      <c r="B202" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C202" t="inlineStr">
-        <is>
-          <t>KN04 - KOBE SUPERCINES ORELLANA</t>
-        </is>
-      </c>
-      <c r="D202" t="inlineStr">
-        <is>
-          <t>MARZO</t>
-        </is>
-      </c>
-      <c r="E202" t="n">
-        <v>3</v>
-      </c>
-      <c r="F202" t="n">
-        <v>26</v>
-      </c>
-      <c r="G202" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="H202" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="I202" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J202" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>KN005</t>
-        </is>
-      </c>
-      <c r="B203" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C203" t="inlineStr">
-        <is>
-          <t>KN05 - KOBE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="D203" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="E203" t="n">
-        <v>2</v>
-      </c>
-      <c r="F203" t="n">
-        <v>24</v>
-      </c>
-      <c r="G203" t="n">
-        <v>54.8</v>
-      </c>
-      <c r="H203" t="n">
-        <v>54.8</v>
-      </c>
-      <c r="I203" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J203" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="inlineStr">
-        <is>
-          <t>KN006</t>
-        </is>
-      </c>
-      <c r="B204" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C204" t="inlineStr">
-        <is>
-          <t>KN06 - KOBE PLAZA BATAN</t>
-        </is>
-      </c>
-      <c r="D204" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="E204" t="n">
-        <v>3</v>
-      </c>
-      <c r="F204" t="n">
-        <v>28</v>
-      </c>
-      <c r="G204" t="n">
-        <v>64.59999999999999</v>
-      </c>
-      <c r="H204" t="n">
-        <v>64.59999999999999</v>
-      </c>
-      <c r="I204" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J204" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="inlineStr">
-        <is>
-          <t>KN007</t>
-        </is>
-      </c>
-      <c r="B205" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C205" t="inlineStr">
-        <is>
-          <t>KN07 - KOBE MALL DEL NORTE</t>
-        </is>
-      </c>
-      <c r="D205" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="E205" t="n">
-        <v>3</v>
-      </c>
-      <c r="F205" t="n">
-        <v>26</v>
-      </c>
-      <c r="G205" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="H205" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="I205" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J205" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>KN008</t>
-        </is>
-      </c>
-      <c r="B206" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C206" t="inlineStr">
-        <is>
-          <t>KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="D206" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="E206" t="n">
-        <v>5</v>
-      </c>
-      <c r="F206" t="n">
-        <v>42</v>
-      </c>
-      <c r="G206" t="n">
-        <v>81.09999999999999</v>
-      </c>
-      <c r="H206" t="n">
-        <v>81.09999999999999</v>
-      </c>
-      <c r="I206" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J206" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>KN009</t>
-        </is>
-      </c>
-      <c r="B207" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C207" t="inlineStr">
-        <is>
-          <t>KN09 - KOBE PLAZA TIA JOYA</t>
-        </is>
-      </c>
-      <c r="D207" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="E207" t="n">
-        <v>3</v>
-      </c>
-      <c r="F207" t="n">
-        <v>26</v>
-      </c>
-      <c r="G207" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="H207" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="I207" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J207" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>KN010</t>
-        </is>
-      </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C208" t="inlineStr">
-        <is>
-          <t>KN10 - KOBE BAMBOO PLAZA VIA A LA C</t>
-        </is>
-      </c>
-      <c r="D208" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="E208" t="n">
-        <v>3</v>
-      </c>
-      <c r="F208" t="n">
-        <v>24</v>
-      </c>
-      <c r="G208" t="n">
-        <v>54</v>
-      </c>
-      <c r="H208" t="n">
-        <v>54</v>
-      </c>
-      <c r="I208" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J208" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>KN011</t>
-        </is>
-      </c>
-      <c r="B209" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C209" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="D209" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="E209" t="n">
-        <v>8</v>
-      </c>
-      <c r="F209" t="n">
-        <v>56</v>
-      </c>
-      <c r="G209" t="n">
-        <v>133.2</v>
-      </c>
-      <c r="H209" t="n">
-        <v>133.2</v>
-      </c>
-      <c r="I209" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J209" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="inlineStr">
-        <is>
-          <t>KN012</t>
-        </is>
-      </c>
-      <c r="B210" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C210" t="inlineStr">
-        <is>
-          <t>KN12 - KOBE RIOC ENTRE RIOS</t>
-        </is>
-      </c>
-      <c r="D210" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="E210" t="n">
-        <v>3</v>
-      </c>
-      <c r="F210" t="n">
-        <v>26</v>
-      </c>
-      <c r="G210" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="H210" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="I210" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J210" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>KN013</t>
-        </is>
-      </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="C211" t="inlineStr">
-        <is>
-          <t>KN13 - KOBE RIOC CEIBOS</t>
-        </is>
-      </c>
-      <c r="D211" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="E211" t="n">
-        <v>3</v>
-      </c>
-      <c r="F211" t="n">
-        <v>26</v>
-      </c>
-      <c r="G211" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="H211" t="n">
-        <v>59.3</v>
-      </c>
-      <c r="I211" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J211" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -26670,7 +26150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1450"/>
+  <dimension ref="A1:J1326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -69835,4188 +69315,18 @@
         <v>9.800000000000001</v>
       </c>
     </row>
-    <row r="1315">
-      <c r="D1315" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1315" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1315" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1315" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1315" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1315" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1315" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1316">
-      <c r="E1316" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1316" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1316" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1316" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1316" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1316" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1317">
-      <c r="D1317" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1317" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1317" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1317" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1317" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1317" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1317" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1318">
-      <c r="D1318" t="inlineStr">
-        <is>
-          <t>GABINETE ENTRADA</t>
-        </is>
-      </c>
-      <c r="E1318" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1318" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1318" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1318" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1318" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1318" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1319">
-      <c r="D1319" t="inlineStr">
-        <is>
-          <t>BODEGA</t>
-        </is>
-      </c>
-      <c r="E1319" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1319" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1319" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1319" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1319" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1319" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1320">
-      <c r="A1320" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="F1320" t="inlineStr">
-        <is>
-          <t>6 ext.</t>
-        </is>
-      </c>
-      <c r="G1320" t="n">
-        <v>40</v>
-      </c>
-      <c r="H1320" t="n">
-        <v>94</v>
-      </c>
-    </row>
+    <row r="1315"/>
+    <row r="1316"/>
+    <row r="1317"/>
+    <row r="1318"/>
+    <row r="1319"/>
+    <row r="1320"/>
     <row r="1321"/>
-    <row r="1322">
-      <c r="D1322" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1322" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1322" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1322" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1322" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1322" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1322" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1323">
-      <c r="D1323" t="inlineStr">
-        <is>
-          <t>BODEGA</t>
-        </is>
-      </c>
-      <c r="E1323" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1323" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1323" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1323" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1323" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1323" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1324">
-      <c r="D1324" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1324" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1324" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1324" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1324" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1324" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1324" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1325">
-      <c r="A1325" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN02 - NOE BOCCA SAMBO</t>
-        </is>
-      </c>
-      <c r="F1325" t="inlineStr">
-        <is>
-          <t>4 ext.</t>
-        </is>
-      </c>
-      <c r="G1325" t="n">
-        <v>32</v>
-      </c>
-      <c r="H1325" t="n">
-        <v>74.40000000000001</v>
-      </c>
-    </row>
+    <row r="1322"/>
+    <row r="1323"/>
+    <row r="1324"/>
+    <row r="1325"/>
     <row r="1326"/>
-    <row r="1327">
-      <c r="D1327" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1327" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1327" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1327" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1327" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1327" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1327" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1328">
-      <c r="D1328" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1328" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1328" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1328" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1328" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1328" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1328" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1329">
-      <c r="D1329" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1329" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1329" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1329" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1329" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1329" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1329" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1330">
-      <c r="D1330" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1330" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1330" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1330" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1330" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1330" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1330" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1331">
-      <c r="D1331" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1331" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1331" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1331" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1331" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1331" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1331" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1332">
-      <c r="D1332" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1332" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1332" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1332" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1332" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1332" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1332" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1333">
-      <c r="D1333" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1333" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1333" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1333" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1333" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1333" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1333" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1334">
-      <c r="D1334" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1334" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1334" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1334" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1334" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1334" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1334" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1335">
-      <c r="D1335" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1335" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1335" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1335" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1335" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1335" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1335" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1336">
-      <c r="D1336" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1336" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1336" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1336" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1336" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="I1336" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1336" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1337">
-      <c r="D1337" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1337" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1337" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1337" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1337" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="I1337" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1337" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1338">
-      <c r="D1338" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1338" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1338" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1338" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1338" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1338" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1338" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1339">
-      <c r="D1339" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1339" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1339" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1339" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1339" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1339" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1339" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1340">
-      <c r="D1340" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1340" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1340" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1340" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1340" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1340" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1340" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1341">
-      <c r="D1341" t="inlineStr">
-        <is>
-          <t>PLANTA</t>
-        </is>
-      </c>
-      <c r="E1341" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1341" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1341" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1341" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1341" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1341" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1342">
-      <c r="A1342" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="F1342" t="inlineStr">
-        <is>
-          <t>16 ext.</t>
-        </is>
-      </c>
-      <c r="G1342" t="n">
-        <v>78</v>
-      </c>
-      <c r="H1342" t="n">
-        <v>181.9</v>
-      </c>
-    </row>
-    <row r="1343"/>
-    <row r="1344">
-      <c r="D1344" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1344" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1344" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1344" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1344" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1344" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1344" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1345">
-      <c r="D1345" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1345" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1345" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1345" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1345" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1345" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1345" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1346">
-      <c r="A1346" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN04 - KOBE SUPERCINES ORELLANA</t>
-        </is>
-      </c>
-      <c r="F1346" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1346" t="n">
-        <v>26</v>
-      </c>
-      <c r="H1346" t="n">
-        <v>59.3</v>
-      </c>
-    </row>
-    <row r="1347"/>
-    <row r="1348">
-      <c r="D1348" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1348" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1348" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1348" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1348" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1348" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1348" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1349">
-      <c r="A1349" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN05 - KOBE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="F1349" t="inlineStr">
-        <is>
-          <t>2 ext.</t>
-        </is>
-      </c>
-      <c r="G1349" t="n">
-        <v>24</v>
-      </c>
-      <c r="H1349" t="n">
-        <v>54.8</v>
-      </c>
-    </row>
-    <row r="1350"/>
-    <row r="1351">
-      <c r="D1351" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1351" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1351" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1351" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1351" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1351" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1351" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1352">
-      <c r="D1352" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1352" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1352" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1352" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1352" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1352" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1352" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1353">
-      <c r="A1353" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN06 - KOBE PLAZA BATAN</t>
-        </is>
-      </c>
-      <c r="F1353" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1353" t="n">
-        <v>28</v>
-      </c>
-      <c r="H1353" t="n">
-        <v>64.59999999999999</v>
-      </c>
-    </row>
-    <row r="1354"/>
-    <row r="1355">
-      <c r="D1355" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1355" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1355" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1355" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1355" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1355" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1355" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1356">
-      <c r="D1356" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1356" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1356" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1356" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1356" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1356" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1356" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1357">
-      <c r="A1357" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN07 - KOBE MALL DEL NORTE</t>
-        </is>
-      </c>
-      <c r="F1357" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1357" t="n">
-        <v>26</v>
-      </c>
-      <c r="H1357" t="n">
-        <v>59.3</v>
-      </c>
-    </row>
-    <row r="1358"/>
-    <row r="1359">
-      <c r="D1359" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1359" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1359" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1359" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1359" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1359" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1359" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1360">
-      <c r="D1360" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1360" t="inlineStr">
-        <is>
-          <t>TIPO K</t>
-        </is>
-      </c>
-      <c r="F1360" t="inlineStr">
-        <is>
-          <t>2.5 GLS</t>
-        </is>
-      </c>
-      <c r="G1360" t="n">
-        <v>12</v>
-      </c>
-      <c r="H1360" t="n">
-        <v>12</v>
-      </c>
-      <c r="I1360" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1360" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1361">
-      <c r="D1361" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1361" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1361" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1361" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1361" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1361" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1361" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1362">
-      <c r="D1362" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1362" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1362" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1362" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1362" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1362" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1362" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1363">
-      <c r="A1363" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="F1363" t="inlineStr">
-        <is>
-          <t>5 ext.</t>
-        </is>
-      </c>
-      <c r="G1363" t="n">
-        <v>42</v>
-      </c>
-      <c r="H1363" t="n">
-        <v>81.09999999999999</v>
-      </c>
-    </row>
-    <row r="1364"/>
-    <row r="1365">
-      <c r="D1365" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1365" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1365" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1365" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1365" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1365" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1365" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1366">
-      <c r="D1366" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1366" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1366" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1366" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1366" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1366" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1366" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1367">
-      <c r="A1367" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN09 - KOBE PLAZA TIA JOYA</t>
-        </is>
-      </c>
-      <c r="F1367" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1367" t="n">
-        <v>26</v>
-      </c>
-      <c r="H1367" t="n">
-        <v>59.3</v>
-      </c>
-    </row>
-    <row r="1368"/>
-    <row r="1369">
-      <c r="D1369" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1369" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1369" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1369" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1369" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1369" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1369" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1370">
-      <c r="D1370" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1370" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1370" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1370" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1370" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1370" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1370" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1371">
-      <c r="A1371" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN10 - KOBE BAMBOO PLAZA VIA A LA C</t>
-        </is>
-      </c>
-      <c r="F1371" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1371" t="n">
-        <v>24</v>
-      </c>
-      <c r="H1371" t="n">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="1372"/>
-    <row r="1373">
-      <c r="D1373" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1373" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1373" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1373" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1373" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="I1373" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1373" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1374">
-      <c r="D1374" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1374" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1374" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1374" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1374" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="I1374" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1374" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1375">
-      <c r="D1375" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1375" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1375" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1375" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1375" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1375" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1375" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1376">
-      <c r="D1376" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1376" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1376" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1376" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1376" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1376" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1376" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1377">
-      <c r="D1377" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1377" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1377" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1377" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1377" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1377" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1377" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1378">
-      <c r="D1378" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1378" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1378" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1378" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1378" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1378" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1378" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1379">
-      <c r="D1379" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1379" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1379" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1379" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1379" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1379" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1379" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1380">
-      <c r="A1380" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="F1380" t="inlineStr">
-        <is>
-          <t>8 ext.</t>
-        </is>
-      </c>
-      <c r="G1380" t="n">
-        <v>56</v>
-      </c>
-      <c r="H1380" t="n">
-        <v>133.2</v>
-      </c>
-    </row>
-    <row r="1381"/>
-    <row r="1382">
-      <c r="D1382" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1382" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1382" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1382" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1382" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1382" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1382" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1383">
-      <c r="D1383" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1383" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1383" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1383" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1383" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1383" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1383" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1384">
-      <c r="A1384" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN12 - KOBE RIOC ENTRE RIOS</t>
-        </is>
-      </c>
-      <c r="F1384" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1384" t="n">
-        <v>26</v>
-      </c>
-      <c r="H1384" t="n">
-        <v>59.3</v>
-      </c>
-    </row>
-    <row r="1385"/>
-    <row r="1386">
-      <c r="D1386" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1386" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1386" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1386" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1386" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1386" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1386" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1387">
-      <c r="D1387" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1387" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1387" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1387" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1387" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1387" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1387" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1388">
-      <c r="A1388" t="inlineStr">
-        <is>
-          <t>TOTALES  SUSHICORP – KN13 - KOBE RIOC CEIBOS</t>
-        </is>
-      </c>
-      <c r="F1388" t="inlineStr">
-        <is>
-          <t>3 ext.</t>
-        </is>
-      </c>
-      <c r="G1388" t="n">
-        <v>26</v>
-      </c>
-      <c r="H1388" t="n">
-        <v>59.3</v>
-      </c>
-    </row>
-    <row r="1389">
-      <c r="A1389" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1389" t="inlineStr">
-        <is>
-          <t>KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1389" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1389" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1389" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1389" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1389" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1389" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1389" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1389" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1390">
-      <c r="A1390" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1390" t="inlineStr">
-        <is>
-          <t>KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1390" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1390" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1390" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1390" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1390" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1390" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1390" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1390" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1391">
-      <c r="A1391" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1391" t="inlineStr">
-        <is>
-          <t>KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1391" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1391" t="inlineStr">
-        <is>
-          <t>OFICINA</t>
-        </is>
-      </c>
-      <c r="E1391" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1391" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1391" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1391" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1391" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1391" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1392">
-      <c r="A1392" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1392" t="inlineStr">
-        <is>
-          <t>KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1392" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1392" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1392" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1392" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1392" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1392" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1392" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1392" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1393">
-      <c r="A1393" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1393" t="inlineStr">
-        <is>
-          <t>KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1393" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1393" t="inlineStr">
-        <is>
-          <t>GABINETE ENTRADA PRINCIPAÑ</t>
-        </is>
-      </c>
-      <c r="E1393" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1393" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1393" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1393" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1393" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1393" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1394">
-      <c r="A1394" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1394" t="inlineStr">
-        <is>
-          <t>KN01 - NOE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1394" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1394" t="inlineStr">
-        <is>
-          <t>BODEGA P/B</t>
-        </is>
-      </c>
-      <c r="E1394" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1394" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1394" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1394" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1394" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1394" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1395">
-      <c r="A1395" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1395" t="inlineStr">
-        <is>
-          <t>KN02 - NOE BOCCA SAMBO</t>
-        </is>
-      </c>
-      <c r="C1395" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1395" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1395" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1395" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1395" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1395" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1395" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1395" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1396">
-      <c r="A1396" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1396" t="inlineStr">
-        <is>
-          <t>KN02 - NOE BOCCA SAMBO</t>
-        </is>
-      </c>
-      <c r="C1396" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1396" t="inlineStr">
-        <is>
-          <t>SALON</t>
-        </is>
-      </c>
-      <c r="E1396" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1396" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1396" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1396" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1396" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1396" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1397">
-      <c r="A1397" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1397" t="inlineStr">
-        <is>
-          <t>KN02 - NOE BOCCA SAMBO</t>
-        </is>
-      </c>
-      <c r="C1397" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1397" t="inlineStr">
-        <is>
-          <t>BODEGA</t>
-        </is>
-      </c>
-      <c r="E1397" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1397" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1397" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1397" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1397" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1397" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1398">
-      <c r="A1398" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1398" t="inlineStr">
-        <is>
-          <t>KN02 - NOE BOCCA SAMBO</t>
-        </is>
-      </c>
-      <c r="C1398" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1398" t="inlineStr">
-        <is>
-          <t>COCINA</t>
-        </is>
-      </c>
-      <c r="E1398" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1398" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1398" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1398" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1398" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1398" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1399">
-      <c r="A1399" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1399" t="inlineStr">
-        <is>
-          <t>KN04 - KOBE SUPERCINES ORELLANA</t>
-        </is>
-      </c>
-      <c r="C1399" t="inlineStr">
-        <is>
-          <t>MARZO</t>
-        </is>
-      </c>
-      <c r="D1399" t="inlineStr"/>
-      <c r="E1399" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1399" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1399" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1399" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1399" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1399" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1400">
-      <c r="A1400" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1400" t="inlineStr">
-        <is>
-          <t>KN04 - KOBE SUPERCINES ORELLANA</t>
-        </is>
-      </c>
-      <c r="C1400" t="inlineStr">
-        <is>
-          <t>MARZO</t>
-        </is>
-      </c>
-      <c r="D1400" t="inlineStr"/>
-      <c r="E1400" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1400" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1400" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1400" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1400" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1400" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1401">
-      <c r="A1401" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1401" t="inlineStr">
-        <is>
-          <t>KN04 - KOBE SUPERCINES ORELLANA</t>
-        </is>
-      </c>
-      <c r="C1401" t="inlineStr">
-        <is>
-          <t>MARZO</t>
-        </is>
-      </c>
-      <c r="D1401" t="inlineStr"/>
-      <c r="E1401" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1401" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1401" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1401" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1401" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1401" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1402">
-      <c r="A1402" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1402" t="inlineStr">
-        <is>
-          <t>KN06 - KOBE PLAZA BATAN</t>
-        </is>
-      </c>
-      <c r="C1402" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1402" t="inlineStr"/>
-      <c r="E1402" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1402" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1402" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1402" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1402" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1402" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1403">
-      <c r="A1403" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1403" t="inlineStr">
-        <is>
-          <t>KN06 - KOBE PLAZA BATAN</t>
-        </is>
-      </c>
-      <c r="C1403" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1403" t="inlineStr"/>
-      <c r="E1403" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1403" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1403" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1403" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1403" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1403" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1404">
-      <c r="A1404" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1404" t="inlineStr">
-        <is>
-          <t>KN06 - KOBE PLAZA BATAN</t>
-        </is>
-      </c>
-      <c r="C1404" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1404" t="inlineStr"/>
-      <c r="E1404" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1404" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1404" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1404" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1404" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1404" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1405">
-      <c r="A1405" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1405" t="inlineStr">
-        <is>
-          <t>KN05 - KOBE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1405" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1405" t="inlineStr"/>
-      <c r="E1405" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1405" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1405" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1405" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1405" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1405" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1406">
-      <c r="A1406" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1406" t="inlineStr">
-        <is>
-          <t>KN05 - KOBE MALL DEL SOL</t>
-        </is>
-      </c>
-      <c r="C1406" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1406" t="inlineStr"/>
-      <c r="E1406" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1406" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1406" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1406" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1406" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1406" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1407">
-      <c r="A1407" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1407" t="inlineStr">
-        <is>
-          <t>KN07 - KOBE MALL DEL NORTE</t>
-        </is>
-      </c>
-      <c r="C1407" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1407" t="inlineStr"/>
-      <c r="E1407" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1407" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1407" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1407" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1407" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1407" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1408">
-      <c r="A1408" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1408" t="inlineStr">
-        <is>
-          <t>KN07 - KOBE MALL DEL NORTE</t>
-        </is>
-      </c>
-      <c r="C1408" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1408" t="inlineStr"/>
-      <c r="E1408" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1408" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1408" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1408" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1408" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1408" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1409">
-      <c r="A1409" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1409" t="inlineStr">
-        <is>
-          <t>KN07 - KOBE MALL DEL NORTE</t>
-        </is>
-      </c>
-      <c r="C1409" t="inlineStr">
-        <is>
-          <t>AGOSTO</t>
-        </is>
-      </c>
-      <c r="D1409" t="inlineStr"/>
-      <c r="E1409" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1409" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1409" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1409" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1409" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1409" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1410">
-      <c r="A1410" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1410" t="inlineStr">
-        <is>
-          <t>KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="C1410" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1410" t="inlineStr"/>
-      <c r="E1410" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1410" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1410" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1410" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1410" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1410" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1411">
-      <c r="A1411" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1411" t="inlineStr">
-        <is>
-          <t>KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="C1411" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1411" t="inlineStr"/>
-      <c r="E1411" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1411" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1411" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1411" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1411" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1411" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1412">
-      <c r="A1412" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1412" t="inlineStr">
-        <is>
-          <t>KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="C1412" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1412" t="inlineStr"/>
-      <c r="E1412" t="inlineStr">
-        <is>
-          <t>TIPO K</t>
-        </is>
-      </c>
-      <c r="F1412" t="inlineStr">
-        <is>
-          <t>2.5 GLS</t>
-        </is>
-      </c>
-      <c r="G1412" t="n">
-        <v>12</v>
-      </c>
-      <c r="H1412" t="n">
-        <v>12</v>
-      </c>
-      <c r="I1412" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1412" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1413">
-      <c r="A1413" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1413" t="inlineStr">
-        <is>
-          <t>KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="C1413" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1413" t="inlineStr"/>
-      <c r="E1413" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1413" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1413" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1413" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1413" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1413" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1414">
-      <c r="A1414" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1414" t="inlineStr">
-        <is>
-          <t>KN08 - NOE SAN MARINO</t>
-        </is>
-      </c>
-      <c r="C1414" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1414" t="inlineStr"/>
-      <c r="E1414" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1414" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1414" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1414" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1414" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1414" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1415">
-      <c r="A1415" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1415" t="inlineStr">
-        <is>
-          <t>KN09 - KOBE PLAZA TIA JOYA</t>
-        </is>
-      </c>
-      <c r="C1415" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1415" t="inlineStr"/>
-      <c r="E1415" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1415" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1415" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1415" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1415" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1415" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1416">
-      <c r="A1416" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1416" t="inlineStr">
-        <is>
-          <t>KN09 - KOBE PLAZA TIA JOYA</t>
-        </is>
-      </c>
-      <c r="C1416" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1416" t="inlineStr"/>
-      <c r="E1416" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1416" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1416" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1416" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1416" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1416" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1417">
-      <c r="A1417" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1417" t="inlineStr">
-        <is>
-          <t>KN09 - KOBE PLAZA TIA JOYA</t>
-        </is>
-      </c>
-      <c r="C1417" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1417" t="inlineStr"/>
-      <c r="E1417" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1417" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1417" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1417" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1417" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1417" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1418">
-      <c r="A1418" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1418" t="inlineStr">
-        <is>
-          <t>KN10 - KOBE BAMBOO PLAZA VIA A LA C</t>
-        </is>
-      </c>
-      <c r="C1418" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1418" t="inlineStr"/>
-      <c r="E1418" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1418" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1418" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1418" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1418" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1418" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1419">
-      <c r="A1419" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1419" t="inlineStr">
-        <is>
-          <t>KN10 - KOBE BAMBOO PLAZA VIA A LA C</t>
-        </is>
-      </c>
-      <c r="C1419" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1419" t="inlineStr"/>
-      <c r="E1419" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1419" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1419" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1419" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1419" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1419" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1420">
-      <c r="A1420" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1420" t="inlineStr">
-        <is>
-          <t>KN10 - KOBE BAMBOO PLAZA VIA A LA C</t>
-        </is>
-      </c>
-      <c r="C1420" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1420" t="inlineStr"/>
-      <c r="E1420" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1420" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1420" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1420" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1420" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1420" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1421">
-      <c r="A1421" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1421" t="inlineStr">
-        <is>
-          <t>KN12 - KOBE RIOC ENTRE RIOS</t>
-        </is>
-      </c>
-      <c r="C1421" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1421" t="inlineStr"/>
-      <c r="E1421" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1421" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1421" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1421" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1421" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1421" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1422">
-      <c r="A1422" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1422" t="inlineStr">
-        <is>
-          <t>KN12 - KOBE RIOC ENTRE RIOS</t>
-        </is>
-      </c>
-      <c r="C1422" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1422" t="inlineStr"/>
-      <c r="E1422" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1422" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1422" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1422" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1422" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1422" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1423">
-      <c r="A1423" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1423" t="inlineStr">
-        <is>
-          <t>KN12 - KOBE RIOC ENTRE RIOS</t>
-        </is>
-      </c>
-      <c r="C1423" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1423" t="inlineStr"/>
-      <c r="E1423" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1423" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1423" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1423" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1423" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1423" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1424">
-      <c r="A1424" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1424" t="inlineStr">
-        <is>
-          <t>KN13 - KOBE RIOC CEIBOS</t>
-        </is>
-      </c>
-      <c r="C1424" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1424" t="inlineStr"/>
-      <c r="E1424" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1424" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1424" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1424" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1424" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1424" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1425">
-      <c r="A1425" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1425" t="inlineStr">
-        <is>
-          <t>KN13 - KOBE RIOC CEIBOS</t>
-        </is>
-      </c>
-      <c r="C1425" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1425" t="inlineStr"/>
-      <c r="E1425" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1425" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1425" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1425" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1425" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1425" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1426">
-      <c r="A1426" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1426" t="inlineStr">
-        <is>
-          <t>KN13 - KOBE RIOC CEIBOS</t>
-        </is>
-      </c>
-      <c r="C1426" t="inlineStr">
-        <is>
-          <t>DICIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1426" t="inlineStr"/>
-      <c r="E1426" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1426" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1426" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1426" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1426" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1426" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1427">
-      <c r="A1427" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1427" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1427" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1427" t="inlineStr"/>
-      <c r="E1427" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1427" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1427" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1427" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1427" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1427" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1428">
-      <c r="A1428" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1428" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1428" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1428" t="inlineStr"/>
-      <c r="E1428" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1428" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1428" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1428" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="I1428" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1428" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1429">
-      <c r="A1429" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1429" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1429" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1429" t="inlineStr"/>
-      <c r="E1429" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1429" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1429" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1429" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="I1429" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1429" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1430">
-      <c r="A1430" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1430" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1430" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1430" t="inlineStr"/>
-      <c r="E1430" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1430" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1430" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1430" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1430" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1430" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1431">
-      <c r="A1431" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1431" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1431" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1431" t="inlineStr"/>
-      <c r="E1431" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1431" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1431" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1431" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1431" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1431" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1432">
-      <c r="A1432" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1432" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1432" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1432" t="inlineStr"/>
-      <c r="E1432" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1432" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1432" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1432" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1432" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1432" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1433">
-      <c r="A1433" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1433" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1433" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1433" t="inlineStr"/>
-      <c r="E1433" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1433" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1433" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1433" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1433" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1433" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1434">
-      <c r="A1434" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1434" t="inlineStr">
-        <is>
-          <t>KN11 - KOBE URDESA</t>
-        </is>
-      </c>
-      <c r="C1434" t="inlineStr">
-        <is>
-          <t>NOVIEMBRE</t>
-        </is>
-      </c>
-      <c r="D1434" t="inlineStr"/>
-      <c r="E1434" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1434" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1434" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1434" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1434" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1434" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1435">
-      <c r="A1435" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1435" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1435" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1435" t="inlineStr"/>
-      <c r="E1435" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1435" t="inlineStr">
-        <is>
-          <t>50 LBS</t>
-        </is>
-      </c>
-      <c r="G1435" t="n">
-        <v>20</v>
-      </c>
-      <c r="H1435" t="n">
-        <v>45</v>
-      </c>
-      <c r="I1435" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1435" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1436">
-      <c r="A1436" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1436" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1436" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1436" t="inlineStr"/>
-      <c r="E1436" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1436" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1436" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1436" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1436" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1436" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1437">
-      <c r="A1437" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1437" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1437" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1437" t="inlineStr"/>
-      <c r="E1437" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1437" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1437" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1437" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1437" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1437" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1438">
-      <c r="A1438" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1438" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1438" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1438" t="inlineStr"/>
-      <c r="E1438" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1438" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1438" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1438" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1438" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1438" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1439">
-      <c r="A1439" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1439" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1439" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1439" t="inlineStr"/>
-      <c r="E1439" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1439" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1439" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1439" t="n">
-        <v>9</v>
-      </c>
-      <c r="I1439" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1439" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1440">
-      <c r="A1440" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1440" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1440" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1440" t="inlineStr"/>
-      <c r="E1440" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1440" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1440" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1440" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1440" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1440" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1441">
-      <c r="A1441" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1441" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1441" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1441" t="inlineStr"/>
-      <c r="E1441" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1441" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1441" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1441" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1441" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1441" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1442">
-      <c r="A1442" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1442" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1442" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1442" t="inlineStr"/>
-      <c r="E1442" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1442" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1442" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1442" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1442" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1442" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1443">
-      <c r="A1443" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1443" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1443" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1443" t="inlineStr"/>
-      <c r="E1443" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1443" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1443" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1443" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1443" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1443" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1444">
-      <c r="A1444" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1444" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1444" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1444" t="inlineStr"/>
-      <c r="E1444" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="F1444" t="inlineStr">
-        <is>
-          <t>5 LBS</t>
-        </is>
-      </c>
-      <c r="G1444" t="n">
-        <v>2</v>
-      </c>
-      <c r="H1444" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I1444" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1444" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1445">
-      <c r="A1445" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1445" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1445" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1445" t="inlineStr"/>
-      <c r="E1445" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1445" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1445" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1445" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="I1445" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1445" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1446">
-      <c r="A1446" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1446" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1446" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1446" t="inlineStr"/>
-      <c r="E1446" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1446" t="inlineStr">
-        <is>
-          <t>20 LBS</t>
-        </is>
-      </c>
-      <c r="G1446" t="n">
-        <v>8</v>
-      </c>
-      <c r="H1446" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="I1446" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1446" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1447">
-      <c r="A1447" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1447" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1447" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1447" t="inlineStr"/>
-      <c r="E1447" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1447" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1447" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1447" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1447" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1447" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1448">
-      <c r="A1448" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1448" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1448" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1448" t="inlineStr"/>
-      <c r="E1448" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1448" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1448" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1448" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1448" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1448" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1449">
-      <c r="A1449" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1449" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1449" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1449" t="inlineStr"/>
-      <c r="E1449" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1449" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1449" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1449" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1449" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1449" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="1450">
-      <c r="A1450" t="inlineStr">
-        <is>
-          <t>SUSHICORP</t>
-        </is>
-      </c>
-      <c r="B1450" t="inlineStr">
-        <is>
-          <t>KN03 - KOBE PLANTA</t>
-        </is>
-      </c>
-      <c r="C1450" t="inlineStr">
-        <is>
-          <t>FEBRERO</t>
-        </is>
-      </c>
-      <c r="D1450" t="inlineStr"/>
-      <c r="E1450" t="inlineStr">
-        <is>
-          <t>PQS</t>
-        </is>
-      </c>
-      <c r="F1450" t="inlineStr">
-        <is>
-          <t>10 LBS</t>
-        </is>
-      </c>
-      <c r="G1450" t="n">
-        <v>4</v>
-      </c>
-      <c r="H1450" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="I1450" t="n">
-        <v>2024</v>
-      </c>
-      <c r="J1450" t="n">
-        <v>2026</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>